<commit_message>
fix report and update run_analysis.py
</commit_message>
<xml_diff>
--- a/outputs/round2/summary_tables.xlsx
+++ b/outputs/round2/summary_tables.xlsx
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="F4" s="38" t="n">
-        <v>0.2711950793440543</v>
+        <v>0.2693118659066443</v>
       </c>
     </row>
   </sheetData>
@@ -42318,7 +42318,7 @@
         </is>
       </c>
       <c r="F3" s="37" t="n">
-        <v>4832</v>
+        <v>4835</v>
       </c>
       <c r="G3" s="37" t="n">
         <v>927</v>
@@ -42327,10 +42327,10 @@
         <v>47</v>
       </c>
       <c r="I3" s="38" t="n">
-        <v>60222</v>
+        <v>60324</v>
       </c>
       <c r="J3" s="38" t="n">
-        <v>3258.380493770956</v>
+        <v>3268.845693770956</v>
       </c>
     </row>
     <row r="4">
@@ -42355,7 +42355,7 @@
         </is>
       </c>
       <c r="F4" s="37" t="n">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="G4" s="37" t="n">
         <v>315</v>
@@ -42364,10 +42364,10 @@
         <v>18</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>38208</v>
+        <v>38220</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>2277.344344558934</v>
+        <v>2278.575544558933</v>
       </c>
     </row>
     <row r="5">
@@ -42392,7 +42392,7 @@
         </is>
       </c>
       <c r="F5" s="37" t="n">
-        <v>1105</v>
+        <v>1114</v>
       </c>
       <c r="G5" s="37" t="n">
         <v>230</v>
@@ -42401,10 +42401,10 @@
         <v>10</v>
       </c>
       <c r="I5" s="38" t="n">
-        <v>22975</v>
+        <v>23428</v>
       </c>
       <c r="J5" s="38" t="n">
-        <v>1361.0699681542</v>
+        <v>1407.5477681542</v>
       </c>
     </row>
     <row r="6">
@@ -42429,7 +42429,7 @@
         </is>
       </c>
       <c r="F6" s="37" t="n">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="G6" s="37" t="n">
         <v>207</v>
@@ -42438,10 +42438,10 @@
         <v>8</v>
       </c>
       <c r="I6" s="38" t="n">
-        <v>18658</v>
+        <v>18676</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>1117.554435340917</v>
+        <v>1119.401235340917</v>
       </c>
     </row>
     <row r="7">
@@ -42466,7 +42466,7 @@
         </is>
       </c>
       <c r="F7" s="37" t="n">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="G7" s="37" t="n">
         <v>118</v>
@@ -42475,10 +42475,10 @@
         <v>9</v>
       </c>
       <c r="I7" s="38" t="n">
-        <v>11794</v>
+        <v>11962</v>
       </c>
       <c r="J7" s="38" t="n">
-        <v>708.7796899680001</v>
+        <v>726.0164899680001</v>
       </c>
     </row>
     <row r="8">
@@ -42540,19 +42540,19 @@
         </is>
       </c>
       <c r="F9" s="37" t="n">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="G9" s="37" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H9" s="37" t="n">
         <v>7</v>
       </c>
       <c r="I9" s="38" t="n">
-        <v>11597</v>
+        <v>11644</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>704.6392388626667</v>
+        <v>709.4614388626667</v>
       </c>
     </row>
     <row r="10">
@@ -42614,7 +42614,7 @@
         </is>
       </c>
       <c r="F11" s="37" t="n">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G11" s="37" t="n">
         <v>67</v>
@@ -42623,10 +42623,10 @@
         <v>5</v>
       </c>
       <c r="I11" s="38" t="n">
-        <v>5827</v>
+        <v>5967</v>
       </c>
       <c r="J11" s="38" t="n">
-        <v>289.9722021916667</v>
+        <v>304.3362021916667</v>
       </c>
     </row>
     <row r="12">
@@ -42651,19 +42651,19 @@
         </is>
       </c>
       <c r="F12" s="37" t="n">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G12" s="37" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H12" s="37" t="n">
         <v>4</v>
       </c>
       <c r="I12" s="38" t="n">
-        <v>5359</v>
+        <v>5515</v>
       </c>
       <c r="J12" s="38" t="n">
-        <v>269.9409718833334</v>
+        <v>285.9465718833333</v>
       </c>
     </row>
     <row r="13">
@@ -42799,7 +42799,7 @@
         </is>
       </c>
       <c r="F16" s="37" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G16" s="37" t="n">
         <v>57</v>
@@ -42808,10 +42808,10 @@
         <v>5</v>
       </c>
       <c r="I16" s="38" t="n">
-        <v>4553</v>
+        <v>4565</v>
       </c>
       <c r="J16" s="38" t="n">
-        <v>256.1966613778667</v>
+        <v>257.4278613778667</v>
       </c>
     </row>
     <row r="17">
@@ -42836,7 +42836,7 @@
         </is>
       </c>
       <c r="F17" s="37" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G17" s="37" t="n">
         <v>132</v>
@@ -42845,10 +42845,10 @@
         <v>12</v>
       </c>
       <c r="I17" s="38" t="n">
-        <v>3996</v>
+        <v>4020</v>
       </c>
       <c r="J17" s="38" t="n">
-        <v>182.9311078786667</v>
+        <v>185.3935078786667</v>
       </c>
     </row>
     <row r="18">
@@ -42910,7 +42910,7 @@
         </is>
       </c>
       <c r="F19" s="37" t="n">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G19" s="37" t="n">
         <v>96</v>
@@ -42919,10 +42919,10 @@
         <v>11</v>
       </c>
       <c r="I19" s="38" t="n">
-        <v>3266</v>
+        <v>3278</v>
       </c>
       <c r="J19" s="38" t="n">
-        <v>175.792520484</v>
+        <v>177.023720484</v>
       </c>
     </row>
     <row r="20">
@@ -43021,7 +43021,7 @@
         </is>
       </c>
       <c r="F22" s="37" t="n">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="G22" s="37" t="n">
         <v>54</v>
@@ -43030,10 +43030,10 @@
         <v>6</v>
       </c>
       <c r="I22" s="38" t="n">
-        <v>3064</v>
+        <v>3110</v>
       </c>
       <c r="J22" s="38" t="n">
-        <v>141.342257943</v>
+        <v>146.061857943</v>
       </c>
     </row>
     <row r="23">
@@ -43113,17 +43113,17 @@
     <row r="25">
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Hà Nội</t>
+          <t>Vĩnh Long</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -43132,35 +43132,35 @@
         </is>
       </c>
       <c r="F25" s="37" t="n">
-        <v>399</v>
+        <v>189</v>
       </c>
       <c r="G25" s="37" t="n">
-        <v>135</v>
+        <v>43</v>
       </c>
       <c r="H25" s="37" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>2192.666666666667</v>
+        <v>2200</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>114.8266909098333</v>
+        <v>103.2210027056</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Vĩnh Long</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -43169,19 +43169,19 @@
         </is>
       </c>
       <c r="F26" s="37" t="n">
-        <v>187</v>
+        <v>399</v>
       </c>
       <c r="G26" s="37" t="n">
-        <v>43</v>
+        <v>135</v>
       </c>
       <c r="H26" s="37" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>2168</v>
+        <v>2192.666666666667</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>99.93780270560001</v>
+        <v>114.8266909098333</v>
       </c>
     </row>
     <row r="27">
@@ -43206,7 +43206,7 @@
         </is>
       </c>
       <c r="F27" s="37" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G27" s="37" t="n">
         <v>44</v>
@@ -43215,10 +43215,10 @@
         <v>7</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>2031</v>
+        <v>2067</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>97.16785063433335</v>
+        <v>100.8614506343333</v>
       </c>
     </row>
     <row r="28">
@@ -43243,7 +43243,7 @@
         </is>
       </c>
       <c r="F28" s="37" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="G28" s="37" t="n">
         <v>277</v>
@@ -43252,10 +43252,10 @@
         <v>1</v>
       </c>
       <c r="I28" s="38" t="n">
-        <v>1883</v>
+        <v>1885</v>
       </c>
       <c r="J28" s="38" t="n">
-        <v>89.94904067413691</v>
+        <v>90.04729667413692</v>
       </c>
     </row>
     <row r="29">
@@ -43280,7 +43280,7 @@
         </is>
       </c>
       <c r="F29" s="37" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G29" s="37" t="n">
         <v>28</v>
@@ -43289,10 +43289,10 @@
         <v>3</v>
       </c>
       <c r="I29" s="38" t="n">
-        <v>1324</v>
+        <v>1392</v>
       </c>
       <c r="J29" s="38" t="n">
-        <v>65.52657533333334</v>
+        <v>72.50337533333334</v>
       </c>
     </row>
     <row r="30">
@@ -43354,19 +43354,19 @@
         </is>
       </c>
       <c r="F31" s="37" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G31" s="37" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H31" s="37" t="n">
         <v>2</v>
       </c>
       <c r="I31" s="38" t="n">
-        <v>1022</v>
+        <v>1042</v>
       </c>
       <c r="J31" s="38" t="n">
-        <v>43.73682804166667</v>
+        <v>45.78882804166667</v>
       </c>
     </row>
     <row r="32">
@@ -43391,7 +43391,7 @@
         </is>
       </c>
       <c r="F32" s="37" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G32" s="37" t="n">
         <v>22</v>
@@ -43400,10 +43400,10 @@
         <v>3</v>
       </c>
       <c r="I32" s="38" t="n">
-        <v>997</v>
+        <v>1005</v>
       </c>
       <c r="J32" s="38" t="n">
-        <v>56.93964978291667</v>
+        <v>57.76044978291667</v>
       </c>
     </row>
     <row r="33">
@@ -43502,7 +43502,7 @@
         </is>
       </c>
       <c r="F35" s="37" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G35" s="37" t="n">
         <v>31</v>
@@ -43511,10 +43511,10 @@
         <v>3</v>
       </c>
       <c r="I35" s="38" t="n">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="J35" s="38" t="n">
-        <v>34.5139584146</v>
+        <v>34.9243584146</v>
       </c>
     </row>
     <row r="36">
@@ -46530,7 +46530,7 @@
         </is>
       </c>
       <c r="C3" s="37" t="n">
-        <v>6690</v>
+        <v>6693</v>
       </c>
       <c r="D3" s="37" t="n">
         <v>1402</v>
@@ -46539,10 +46539,10 @@
         <v>87</v>
       </c>
       <c r="F3" s="38" t="n">
-        <v>65425.27638888889</v>
+        <v>65527.27638888889</v>
       </c>
       <c r="G3" s="38" t="n">
-        <v>3548.7060755534</v>
+        <v>3559.1712755534</v>
       </c>
       <c r="H3" s="37" t="n">
         <v>927</v>
@@ -46551,16 +46551,16 @@
         <v>475</v>
       </c>
       <c r="J3" s="38" t="n">
-        <v>60222</v>
+        <v>60324</v>
       </c>
       <c r="K3" s="38" t="n">
         <v>5203.276388888889</v>
       </c>
       <c r="L3" s="38" t="n">
-        <v>0.9204699364514637</v>
+        <v>0.9205937332415791</v>
       </c>
       <c r="M3" s="38" t="n">
-        <v>0.07953006354853635</v>
+        <v>0.07940626675842093</v>
       </c>
       <c r="N3" s="12" t="inlineStr">
         <is>
@@ -46581,7 +46581,7 @@
         </is>
       </c>
       <c r="C4" s="37" t="n">
-        <v>2298</v>
+        <v>2299</v>
       </c>
       <c r="D4" s="37" t="n">
         <v>661</v>
@@ -46590,10 +46590,10 @@
         <v>60</v>
       </c>
       <c r="F4" s="38" t="n">
-        <v>42999.83154761905</v>
+        <v>43011.83154761905</v>
       </c>
       <c r="G4" s="38" t="n">
-        <v>2562.02549514391</v>
+        <v>2563.25669514391</v>
       </c>
       <c r="H4" s="37" t="n">
         <v>315</v>
@@ -46602,16 +46602,16 @@
         <v>346</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>38208</v>
+        <v>38220</v>
       </c>
       <c r="K4" s="38" t="n">
         <v>4791.831547619047</v>
       </c>
       <c r="L4" s="38" t="n">
-        <v>0.8885616204725719</v>
+        <v>0.8885927110006013</v>
       </c>
       <c r="M4" s="38" t="n">
-        <v>0.1114383795274281</v>
+        <v>0.1114072889993987</v>
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
@@ -46632,7 +46632,7 @@
         </is>
       </c>
       <c r="C5" s="37" t="n">
-        <v>1354</v>
+        <v>1356</v>
       </c>
       <c r="D5" s="37" t="n">
         <v>434</v>
@@ -46641,10 +46641,10 @@
         <v>15</v>
       </c>
       <c r="F5" s="38" t="n">
-        <v>6054.083333333333</v>
+        <v>6080.083333333333</v>
       </c>
       <c r="G5" s="38" t="n">
-        <v>281.3840679694703</v>
+        <v>283.9447239694703</v>
       </c>
       <c r="H5" s="37" t="n">
         <v>409</v>
@@ -46653,16 +46653,16 @@
         <v>25</v>
       </c>
       <c r="J5" s="38" t="n">
-        <v>5879</v>
+        <v>5905</v>
       </c>
       <c r="K5" s="38" t="n">
         <v>175.0833333333333</v>
       </c>
       <c r="L5" s="38" t="n">
-        <v>0.9710801249845147</v>
+        <v>0.9712037938076508</v>
       </c>
       <c r="M5" s="38" t="n">
-        <v>0.02891987501548542</v>
+        <v>0.02879620619234934</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
@@ -46683,7 +46683,7 @@
         </is>
       </c>
       <c r="C6" s="37" t="n">
-        <v>1308</v>
+        <v>1317</v>
       </c>
       <c r="D6" s="37" t="n">
         <v>296</v>
@@ -46692,10 +46692,10 @@
         <v>14</v>
       </c>
       <c r="F6" s="38" t="n">
-        <v>23887.47916666667</v>
+        <v>24340.47916666667</v>
       </c>
       <c r="G6" s="38" t="n">
-        <v>1413.726266025034</v>
+        <v>1460.204066025033</v>
       </c>
       <c r="H6" s="37" t="n">
         <v>230</v>
@@ -46704,16 +46704,16 @@
         <v>66</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>22975</v>
+        <v>23428</v>
       </c>
       <c r="K6" s="38" t="n">
         <v>912.4791666666666</v>
       </c>
       <c r="L6" s="38" t="n">
-        <v>0.9618009434859092</v>
+        <v>0.9625118650944114</v>
       </c>
       <c r="M6" s="38" t="n">
-        <v>0.0381990565140908</v>
+        <v>0.03748813490558851</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
@@ -46785,7 +46785,7 @@
         </is>
       </c>
       <c r="C8" s="37" t="n">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="D8" s="37" t="n">
         <v>257</v>
@@ -46794,10 +46794,10 @@
         <v>10</v>
       </c>
       <c r="F8" s="38" t="n">
-        <v>19426.875</v>
+        <v>19444.875</v>
       </c>
       <c r="G8" s="38" t="n">
-        <v>1160.53608698675</v>
+        <v>1162.38288698675</v>
       </c>
       <c r="H8" s="37" t="n">
         <v>207</v>
@@ -46806,16 +46806,16 @@
         <v>50</v>
       </c>
       <c r="J8" s="38" t="n">
-        <v>18658</v>
+        <v>18676</v>
       </c>
       <c r="K8" s="38" t="n">
         <v>768.875</v>
       </c>
       <c r="L8" s="38" t="n">
-        <v>0.9604220956793103</v>
+        <v>0.9604587326994902</v>
       </c>
       <c r="M8" s="38" t="n">
-        <v>0.03957790432068976</v>
+        <v>0.03954126730050977</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
@@ -46836,37 +46836,37 @@
         </is>
       </c>
       <c r="C9" s="37" t="n">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="D9" s="37" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E9" s="37" t="n">
         <v>9</v>
       </c>
       <c r="F9" s="38" t="n">
-        <v>12054.5</v>
+        <v>12101.5</v>
       </c>
       <c r="G9" s="38" t="n">
-        <v>728.852250271</v>
+        <v>733.6744502710001</v>
       </c>
       <c r="H9" s="37" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I9" s="37" t="n">
         <v>43</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>11597</v>
+        <v>11644</v>
       </c>
       <c r="K9" s="38" t="n">
         <v>457.5</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>0.9620473682027458</v>
+        <v>0.9621947692434822</v>
       </c>
       <c r="M9" s="38" t="n">
-        <v>0.03795263179725414</v>
+        <v>0.03780523075651779</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
@@ -46938,7 +46938,7 @@
         </is>
       </c>
       <c r="C11" s="37" t="n">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="D11" s="37" t="n">
         <v>148</v>
@@ -46947,10 +46947,10 @@
         <v>11</v>
       </c>
       <c r="F11" s="38" t="n">
-        <v>12180.95833333333</v>
+        <v>12348.95833333333</v>
       </c>
       <c r="G11" s="38" t="n">
-        <v>727.4485638780001</v>
+        <v>744.6853638780001</v>
       </c>
       <c r="H11" s="37" t="n">
         <v>118</v>
@@ -46959,16 +46959,16 @@
         <v>30</v>
       </c>
       <c r="J11" s="38" t="n">
-        <v>11794</v>
+        <v>11962</v>
       </c>
       <c r="K11" s="38" t="n">
         <v>386.9583333333333</v>
       </c>
       <c r="L11" s="38" t="n">
-        <v>0.9682325213875481</v>
+        <v>0.968664698439477</v>
       </c>
       <c r="M11" s="38" t="n">
-        <v>0.03176747861245181</v>
+        <v>0.03133530156052299</v>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
@@ -47040,7 +47040,7 @@
         </is>
       </c>
       <c r="C13" s="37" t="n">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D13" s="37" t="n">
         <v>128</v>
@@ -47049,10 +47049,10 @@
         <v>14</v>
       </c>
       <c r="F13" s="38" t="n">
-        <v>3366.5</v>
+        <v>3378.5</v>
       </c>
       <c r="G13" s="38" t="n">
-        <v>182.5933075673333</v>
+        <v>183.8245075673333</v>
       </c>
       <c r="H13" s="37" t="n">
         <v>96</v>
@@ -47061,16 +47061,16 @@
         <v>32</v>
       </c>
       <c r="J13" s="38" t="n">
-        <v>3266</v>
+        <v>3278</v>
       </c>
       <c r="K13" s="38" t="n">
         <v>100.5</v>
       </c>
       <c r="L13" s="38" t="n">
-        <v>0.9701470369820289</v>
+        <v>0.970253070889448</v>
       </c>
       <c r="M13" s="38" t="n">
-        <v>0.02985296301797119</v>
+        <v>0.02974692911055202</v>
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
@@ -47142,37 +47142,37 @@
         </is>
       </c>
       <c r="C15" s="37" t="n">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="D15" s="37" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E15" s="37" t="n">
         <v>5</v>
       </c>
       <c r="F15" s="38" t="n">
-        <v>5404.166666666667</v>
+        <v>5560.166666666667</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>276.7181615433333</v>
+        <v>292.7237615433334</v>
       </c>
       <c r="H15" s="37" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I15" s="37" t="n">
         <v>1</v>
       </c>
       <c r="J15" s="38" t="n">
-        <v>5359</v>
+        <v>5515</v>
       </c>
       <c r="K15" s="38" t="n">
         <v>45.16666666666666</v>
       </c>
       <c r="L15" s="38" t="n">
-        <v>0.9916422513492675</v>
+        <v>0.9918767423038877</v>
       </c>
       <c r="M15" s="38" t="n">
-        <v>0.008357748650732459</v>
+        <v>0.008123257696112225</v>
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
@@ -47244,7 +47244,7 @@
         </is>
       </c>
       <c r="C17" s="37" t="n">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D17" s="37" t="n">
         <v>73</v>
@@ -47253,10 +47253,10 @@
         <v>6</v>
       </c>
       <c r="F17" s="38" t="n">
-        <v>5841.75</v>
+        <v>5981.75</v>
       </c>
       <c r="G17" s="38" t="n">
-        <v>291.3835137333334</v>
+        <v>305.7475137333333</v>
       </c>
       <c r="H17" s="37" t="n">
         <v>67</v>
@@ -47265,16 +47265,16 @@
         <v>6</v>
       </c>
       <c r="J17" s="38" t="n">
-        <v>5827</v>
+        <v>5967</v>
       </c>
       <c r="K17" s="38" t="n">
         <v>14.75</v>
       </c>
       <c r="L17" s="38" t="n">
-        <v>0.997475071682287</v>
+        <v>0.9975341664228695</v>
       </c>
       <c r="M17" s="38" t="n">
-        <v>0.002524928317713014</v>
+        <v>0.002465833577130438</v>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
@@ -47396,31 +47396,31 @@
         </is>
       </c>
       <c r="D3" s="37" t="n">
-        <v>885</v>
+        <v>887</v>
       </c>
       <c r="E3" s="37" t="n">
-        <v>3684</v>
+        <v>3715</v>
       </c>
       <c r="F3" s="37" t="n">
         <v>61</v>
       </c>
       <c r="G3" s="38" t="n">
-        <v>65027</v>
+        <v>65993</v>
       </c>
       <c r="H3" s="38" t="n">
-        <v>3640.19896471415</v>
+        <v>3739.31056471415</v>
       </c>
       <c r="I3" s="38" t="n">
-        <v>0.8634146341463415</v>
+        <v>0.8636806231742941</v>
       </c>
       <c r="J3" s="38" t="n">
-        <v>0.9757919625001289</v>
+        <v>0.9761378620498172</v>
       </c>
       <c r="K3" s="38" t="n">
-        <v>0.2279752704791345</v>
+        <v>0.2283140283140283</v>
       </c>
       <c r="L3" s="38" t="n">
-        <v>0.2642450200336467</v>
+        <v>0.2666965721814052</v>
       </c>
     </row>
     <row r="4">
@@ -47450,10 +47450,10 @@
         <v>97.97123456958334</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>0.1365853658536585</v>
+        <v>0.1363193768257059</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>0.02420803749987104</v>
+        <v>0.02386213795018272</v>
       </c>
       <c r="K4" s="38" t="n">
         <v>0.0966183574879227</v>
@@ -47495,10 +47495,10 @@
         <v>0.9686617105211766</v>
       </c>
       <c r="K5" s="38" t="n">
-        <v>0.02421432251416795</v>
+        <v>0.0241956241956242</v>
       </c>
       <c r="L5" s="38" t="n">
-        <v>0.01259722210934389</v>
+        <v>0.01252798590399522</v>
       </c>
     </row>
     <row r="6">
@@ -47552,31 +47552,31 @@
         </is>
       </c>
       <c r="D7" s="37" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E7" s="37" t="n">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="F7" s="37" t="n">
         <v>12</v>
       </c>
       <c r="G7" s="38" t="n">
-        <v>5936</v>
+        <v>5956</v>
       </c>
       <c r="H7" s="38" t="n">
-        <v>292.2876754613334</v>
+        <v>294.3396754613333</v>
       </c>
       <c r="I7" s="38" t="n">
-        <v>0.7967479674796748</v>
+        <v>0.7975708502024291</v>
       </c>
       <c r="J7" s="38" t="n">
-        <v>0.9085714285714286</v>
+        <v>0.9088504577822991</v>
       </c>
       <c r="K7" s="38" t="n">
-        <v>0.05048943843379701</v>
+        <v>0.05070785070785071</v>
       </c>
       <c r="L7" s="38" t="n">
-        <v>0.02412164852937591</v>
+        <v>0.02406989807877274</v>
       </c>
     </row>
     <row r="8">
@@ -47606,10 +47606,10 @@
         <v>39.60646415966666</v>
       </c>
       <c r="I8" s="38" t="n">
-        <v>0.2032520325203252</v>
+        <v>0.2024291497975708</v>
       </c>
       <c r="J8" s="38" t="n">
-        <v>0.09142857142857144</v>
+        <v>0.09114954221770093</v>
       </c>
       <c r="K8" s="38" t="n">
         <v>0.03450655624568668</v>
@@ -47633,28 +47633,28 @@
         <v>1795</v>
       </c>
       <c r="E9" s="37" t="n">
-        <v>7741</v>
+        <v>7750</v>
       </c>
       <c r="F9" s="37" t="n">
         <v>91</v>
       </c>
       <c r="G9" s="38" t="n">
-        <v>116624</v>
+        <v>116932</v>
       </c>
       <c r="H9" s="38" t="n">
-        <v>6544.69359790356</v>
+        <v>6576.18745390356</v>
       </c>
       <c r="I9" s="38" t="n">
         <v>0.6866870696250956</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>0.9168993195731001</v>
+        <v>0.9171000617553824</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>0.4623905203503349</v>
+        <v>0.462033462033462</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>0.4739156229935876</v>
+        <v>0.4725556282986995</v>
       </c>
     </row>
     <row r="10">
@@ -47687,7 +47687,7 @@
         <v>0.3133129303749044</v>
       </c>
       <c r="J10" s="38" t="n">
-        <v>0.0831006804268999</v>
+        <v>0.08289993824461755</v>
       </c>
       <c r="K10" s="38" t="n">
         <v>0.5652173913043478</v>
@@ -47711,28 +47711,28 @@
         <v>670</v>
       </c>
       <c r="E11" s="37" t="n">
-        <v>2850</v>
+        <v>2859</v>
       </c>
       <c r="F11" s="37" t="n">
         <v>56</v>
       </c>
       <c r="G11" s="38" t="n">
-        <v>38490</v>
+        <v>38556</v>
       </c>
       <c r="H11" s="38" t="n">
-        <v>2261.00687915845</v>
+        <v>2267.77847915845</v>
       </c>
       <c r="I11" s="38" t="n">
         <v>0.8375</v>
       </c>
       <c r="J11" s="38" t="n">
-        <v>0.9589466286448661</v>
+        <v>0.9590140233456422</v>
       </c>
       <c r="K11" s="38" t="n">
-        <v>0.1725914477073673</v>
+        <v>0.1724581724581725</v>
       </c>
       <c r="L11" s="38" t="n">
-        <v>0.1564087351576278</v>
+        <v>0.1558158143594966</v>
       </c>
     </row>
     <row r="12">
@@ -47765,7 +47765,7 @@
         <v>0.1625</v>
       </c>
       <c r="J12" s="38" t="n">
-        <v>0.04105337135513393</v>
+        <v>0.04098597665435785</v>
       </c>
       <c r="K12" s="38" t="n">
         <v>0.08971704623878538</v>
@@ -47807,10 +47807,10 @@
         <v>0.7674680510049218</v>
       </c>
       <c r="K13" s="38" t="n">
-        <v>0.06233900051519835</v>
+        <v>0.06229086229086229</v>
       </c>
       <c r="L13" s="38" t="n">
-        <v>0.06871175117641801</v>
+        <v>0.06833410117763067</v>
       </c>
     </row>
     <row r="14">
@@ -48019,34 +48019,34 @@
         </is>
       </c>
       <c r="C4" s="37" t="n">
-        <v>3776</v>
+        <v>3782</v>
       </c>
       <c r="D4" s="37" t="n">
         <v>264</v>
       </c>
       <c r="E4" s="38" t="n">
-        <v>40.22329835889158</v>
+        <v>41.32553532606415</v>
       </c>
       <c r="F4" s="38" t="n">
         <v>11</v>
       </c>
       <c r="G4" s="38" t="n">
-        <v>2.057874315830799</v>
+        <v>2.130173049332918</v>
       </c>
       <c r="H4" s="38" t="n">
-        <v>0.53296596725</v>
+        <v>0.5379085</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>4.326800847457627</v>
+        <v>4.333950290851401</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>4.418697033898305</v>
+        <v>4.426493918561608</v>
       </c>
       <c r="K4" s="38" t="n">
-        <v>270.2804347857308</v>
+        <v>270.3707068077138</v>
       </c>
       <c r="L4" s="38" t="n">
-        <v>2.383838383838384</v>
+        <v>2.387626262626263</v>
       </c>
       <c r="M4" s="37" t="n">
         <v>60</v>
@@ -48055,7 +48055,7 @@
         <v>6</v>
       </c>
       <c r="O4" s="38" t="n">
-        <v>0.2711950793440543</v>
+        <v>0.2693118659066443</v>
       </c>
     </row>
   </sheetData>
@@ -48181,7 +48181,7 @@
         <v>75857</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.4994430765500635</v>
+        <v>0.4853506891302162</v>
       </c>
     </row>
     <row r="7">
@@ -48196,10 +48196,10 @@
         </is>
       </c>
       <c r="D7" s="38" t="n">
-        <v>10858.1746031746</v>
+        <v>15268.1746031746</v>
       </c>
       <c r="E7" s="38" t="n">
-        <v>0.07149030583238579</v>
+        <v>0.09768932419435593</v>
       </c>
     </row>
     <row r="8">
@@ -48217,7 +48217,7 @@
         <v>65168</v>
       </c>
       <c r="E8" s="38" t="n">
-        <v>0.4290666176175506</v>
+        <v>0.4169599866754278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: inconsistent report in q1.2 and q1.3; adjust to make sure that geographical interpretation do not include unknown address customers
</commit_message>
<xml_diff>
--- a/outputs/round2/summary_tables.xlsx
+++ b/outputs/round2/summary_tables.xlsx
@@ -48019,34 +48019,34 @@
         </is>
       </c>
       <c r="C4" s="37" t="n">
-        <v>3782</v>
+        <v>3762</v>
       </c>
       <c r="D4" s="37" t="n">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E4" s="38" t="n">
-        <v>41.32553532606415</v>
+        <v>37.66246002210915</v>
       </c>
       <c r="F4" s="38" t="n">
         <v>11</v>
       </c>
       <c r="G4" s="38" t="n">
-        <v>2.130173049332918</v>
+        <v>1.91843572397052</v>
       </c>
       <c r="H4" s="38" t="n">
-        <v>0.5379085</v>
+        <v>0.530985</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>4.333950290851401</v>
+        <v>4.350877192982456</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>4.426493918561608</v>
+        <v>4.443115364167996</v>
       </c>
       <c r="K4" s="38" t="n">
         <v>270.3707068077138</v>
       </c>
       <c r="L4" s="38" t="n">
-        <v>2.387626262626263</v>
+        <v>2.402298850574712</v>
       </c>
       <c r="M4" s="37" t="n">
         <v>60</v>
@@ -48178,10 +48178,10 @@
         </is>
       </c>
       <c r="D6" s="38" t="n">
-        <v>75857</v>
+        <v>68747</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.4853506891302162</v>
+        <v>0.4852061267977776</v>
       </c>
     </row>
     <row r="7">
@@ -48196,10 +48196,10 @@
         </is>
       </c>
       <c r="D7" s="38" t="n">
-        <v>15268.1746031746</v>
+        <v>12218.1746031746</v>
       </c>
       <c r="E7" s="38" t="n">
-        <v>0.09768932419435593</v>
+        <v>0.08623406367907432</v>
       </c>
     </row>
     <row r="8">
@@ -48214,10 +48214,10 @@
         </is>
       </c>
       <c r="D8" s="38" t="n">
-        <v>65168</v>
+        <v>60721</v>
       </c>
       <c r="E8" s="38" t="n">
-        <v>0.4169599866754278</v>
+        <v>0.428559809523148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: fix the false positive parsed customers
</commit_message>
<xml_diff>
--- a/outputs/round2/summary_tables.xlsx
+++ b/outputs/round2/summary_tables.xlsx
@@ -22,8 +22,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Q1.1 Full SKU Ranking'!$B$2:$Q$472</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Q1.1 Monthly Demand'!$B$2:$R$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Q1.1 Class A Deep Dive'!$B$3:$O$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Q1.2 Warehouse by Region'!$B$2:$J$113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Q1.2 Top Provinces'!$B$2:$P$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Q1.2 Warehouse by Region'!$B$2:$J$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Q1.2 Top Provinces'!$B$2:$P$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Q1.2 Warehouse Imbalance'!$B$2:$L$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Q1.3 Segment Profile'!$B$2:$O$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Q1.3 Packaging'!$B$2:$E$8</definedName>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="F4" s="38" t="n">
-        <v>0.2693118659066443</v>
+        <v>0.272943114847685</v>
       </c>
     </row>
   </sheetData>
@@ -42227,7 +42227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J113"/>
+  <dimension ref="B1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -43229,33 +43229,33 @@
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam Bộ</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Đồng Nai</t>
+          <t>Quảng Bình</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>transaction_text_parse</t>
+          <t>distributor_match</t>
         </is>
       </c>
       <c r="F28" s="37" t="n">
-        <v>591</v>
+        <v>101</v>
       </c>
       <c r="G28" s="37" t="n">
-        <v>277</v>
+        <v>28</v>
       </c>
       <c r="H28" s="37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I28" s="38" t="n">
-        <v>1885</v>
+        <v>1392</v>
       </c>
       <c r="J28" s="38" t="n">
-        <v>90.04729667413692</v>
+        <v>72.50337533333334</v>
       </c>
     </row>
     <row r="29">
@@ -43266,12 +43266,12 @@
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Tây Nguyên</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Quảng Bình</t>
+          <t>Lâm Đồng</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -43280,19 +43280,19 @@
         </is>
       </c>
       <c r="F29" s="37" t="n">
-        <v>101</v>
+        <v>386</v>
       </c>
       <c r="G29" s="37" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="H29" s="37" t="n">
         <v>3</v>
       </c>
       <c r="I29" s="38" t="n">
-        <v>1392</v>
+        <v>1075</v>
       </c>
       <c r="J29" s="38" t="n">
-        <v>72.50337533333334</v>
+        <v>42.12744970066667</v>
       </c>
     </row>
     <row r="30">
@@ -43308,7 +43308,7 @@
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Lâm Đồng</t>
+          <t>Gia Lai</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -43317,19 +43317,19 @@
         </is>
       </c>
       <c r="F30" s="37" t="n">
-        <v>386</v>
+        <v>146</v>
       </c>
       <c r="G30" s="37" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="H30" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I30" s="38" t="n">
-        <v>1075</v>
+        <v>1042</v>
       </c>
       <c r="J30" s="38" t="n">
-        <v>42.12744970066667</v>
+        <v>45.78882804166667</v>
       </c>
     </row>
     <row r="31">
@@ -43340,12 +43340,12 @@
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Tây Nguyên</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Gia Lai</t>
+          <t>Quảng Trị</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -43354,25 +43354,25 @@
         </is>
       </c>
       <c r="F31" s="37" t="n">
-        <v>146</v>
+        <v>103</v>
       </c>
       <c r="G31" s="37" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H31" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I31" s="38" t="n">
-        <v>1042</v>
+        <v>1005</v>
       </c>
       <c r="J31" s="38" t="n">
-        <v>45.78882804166667</v>
+        <v>57.76044978291667</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
@@ -43382,7 +43382,7 @@
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Quảng Trị</t>
+          <t>Đà Nẵng</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -43391,19 +43391,19 @@
         </is>
       </c>
       <c r="F32" s="37" t="n">
-        <v>103</v>
+        <v>203</v>
       </c>
       <c r="G32" s="37" t="n">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H32" s="37" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I32" s="38" t="n">
-        <v>1005</v>
+        <v>912.4791666666666</v>
       </c>
       <c r="J32" s="38" t="n">
-        <v>57.76044978291667</v>
+        <v>52.65629787083333</v>
       </c>
     </row>
     <row r="33">
@@ -43414,12 +43414,12 @@
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Đà Nẵng</t>
+          <t>Cần Thơ</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
@@ -43428,25 +43428,25 @@
         </is>
       </c>
       <c r="F33" s="37" t="n">
-        <v>203</v>
+        <v>130</v>
       </c>
       <c r="G33" s="37" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="H33" s="37" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I33" s="38" t="n">
-        <v>912.4791666666666</v>
+        <v>768.875</v>
       </c>
       <c r="J33" s="38" t="n">
-        <v>52.65629787083333</v>
+        <v>42.98165164583333</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -43456,7 +43456,7 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>Cần Thơ</t>
+          <t>Kiên Giang</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -43465,25 +43465,25 @@
         </is>
       </c>
       <c r="F34" s="37" t="n">
-        <v>130</v>
+        <v>191</v>
       </c>
       <c r="G34" s="37" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="H34" s="37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I34" s="38" t="n">
-        <v>768.875</v>
+        <v>716</v>
       </c>
       <c r="J34" s="38" t="n">
-        <v>42.98165164583333</v>
+        <v>34.9243584146</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
@@ -43493,7 +43493,7 @@
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Kiên Giang</t>
+          <t>Tiền Giang</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -43502,35 +43502,35 @@
         </is>
       </c>
       <c r="F35" s="37" t="n">
-        <v>191</v>
+        <v>107</v>
       </c>
       <c r="G35" s="37" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="H35" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" s="38" t="n">
-        <v>716</v>
+        <v>707.5833333333334</v>
       </c>
       <c r="J35" s="38" t="n">
-        <v>34.9243584146</v>
+        <v>36.89416955</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Tiền Giang</t>
+          <t>Phú Yên</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -43539,35 +43539,35 @@
         </is>
       </c>
       <c r="F36" s="37" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="G36" s="37" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="H36" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I36" s="38" t="n">
-        <v>707.5833333333334</v>
+        <v>663</v>
       </c>
       <c r="J36" s="38" t="n">
-        <v>36.89416955</v>
+        <v>30.84612521666667</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Tây Nguyên</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Phú Yên</t>
+          <t>Đắk Lắk</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
@@ -43576,19 +43576,19 @@
         </is>
       </c>
       <c r="F37" s="37" t="n">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="G37" s="37" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="H37" s="37" t="n">
         <v>3</v>
       </c>
       <c r="I37" s="38" t="n">
-        <v>663</v>
+        <v>563.5833333333334</v>
       </c>
       <c r="J37" s="38" t="n">
-        <v>30.84612521666667</v>
+        <v>35.26430709166667</v>
       </c>
     </row>
     <row r="38">
@@ -43599,12 +43599,12 @@
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>Tây Nguyên</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Đắk Lắk</t>
+          <t>Khánh Hòa</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -43613,35 +43613,35 @@
         </is>
       </c>
       <c r="F38" s="37" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G38" s="37" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H38" s="37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I38" s="38" t="n">
-        <v>563.5833333333334</v>
+        <v>457.5</v>
       </c>
       <c r="J38" s="38" t="n">
-        <v>35.26430709166667</v>
+        <v>24.21301140833333</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>Khánh Hòa</t>
+          <t>Long An</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -43650,19 +43650,19 @@
         </is>
       </c>
       <c r="F39" s="37" t="n">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="G39" s="37" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H39" s="37" t="n">
         <v>4</v>
       </c>
       <c r="I39" s="38" t="n">
-        <v>457.5</v>
+        <v>453</v>
       </c>
       <c r="J39" s="38" t="n">
-        <v>24.21301140833333</v>
+        <v>19.659989</v>
       </c>
     </row>
     <row r="40">
@@ -43678,7 +43678,7 @@
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Long An</t>
+          <t>Bến Tre</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -43687,35 +43687,35 @@
         </is>
       </c>
       <c r="F40" s="37" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="G40" s="37" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H40" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I40" s="38" t="n">
-        <v>453</v>
+        <v>392</v>
       </c>
       <c r="J40" s="38" t="n">
-        <v>19.659989</v>
+        <v>17.139357909</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Đông Nam Bộ</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Bến Tre</t>
+          <t>Bà Rịa - Vũng Tàu</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
@@ -43724,35 +43724,35 @@
         </is>
       </c>
       <c r="F41" s="37" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G41" s="37" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H41" s="37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I41" s="38" t="n">
-        <v>392</v>
+        <v>386.9583333333333</v>
       </c>
       <c r="J41" s="38" t="n">
-        <v>17.139357909</v>
+        <v>18.66887391</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam Bộ</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Bà Rịa - Vũng Tàu</t>
+          <t>Cà Mau</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -43761,19 +43761,19 @@
         </is>
       </c>
       <c r="F42" s="37" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G42" s="37" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H42" s="37" t="n">
         <v>5</v>
       </c>
       <c r="I42" s="38" t="n">
-        <v>386.9583333333333</v>
+        <v>311</v>
       </c>
       <c r="J42" s="38" t="n">
-        <v>18.66887391</v>
+        <v>15.84589021666667</v>
       </c>
     </row>
     <row r="43">
@@ -43784,12 +43784,12 @@
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Cà Mau</t>
+          <t>Quảng Ninh</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
@@ -43798,19 +43798,19 @@
         </is>
       </c>
       <c r="F43" s="37" t="n">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="G43" s="37" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H43" s="37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I43" s="38" t="n">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J43" s="38" t="n">
-        <v>15.84589021666667</v>
+        <v>26.96094258333333</v>
       </c>
     </row>
     <row r="44">
@@ -43821,12 +43821,12 @@
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Hải Dương</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -43835,19 +43835,19 @@
         </is>
       </c>
       <c r="F44" s="37" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G44" s="37" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H44" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I44" s="38" t="n">
-        <v>309</v>
+        <v>290</v>
       </c>
       <c r="J44" s="38" t="n">
-        <v>26.96094258333333</v>
+        <v>13.876579</v>
       </c>
     </row>
     <row r="45">
@@ -43858,12 +43858,12 @@
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Hải Dương</t>
+          <t>Đồng Tháp</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
@@ -43872,19 +43872,19 @@
         </is>
       </c>
       <c r="F45" s="37" t="n">
-        <v>11</v>
+        <v>140</v>
       </c>
       <c r="G45" s="37" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="H45" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45" s="38" t="n">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="J45" s="38" t="n">
-        <v>13.876579</v>
+        <v>13.4992490338</v>
       </c>
     </row>
     <row r="46">
@@ -43895,12 +43895,12 @@
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Đông Nam Bộ</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>Đồng Tháp</t>
+          <t>Bình Phước</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -43909,19 +43909,19 @@
         </is>
       </c>
       <c r="F46" s="37" t="n">
-        <v>140</v>
+        <v>37</v>
       </c>
       <c r="G46" s="37" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="H46" s="37" t="n">
         <v>3</v>
       </c>
       <c r="I46" s="38" t="n">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="J46" s="38" t="n">
-        <v>13.4992490338</v>
+        <v>14.74294533333333</v>
       </c>
     </row>
     <row r="47">
@@ -43937,7 +43937,7 @@
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>Bình Phước</t>
+          <t>Tây Ninh</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
@@ -43946,19 +43946,19 @@
         </is>
       </c>
       <c r="F47" s="37" t="n">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="G47" s="37" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H47" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I47" s="38" t="n">
-        <v>273</v>
+        <v>248</v>
       </c>
       <c r="J47" s="38" t="n">
-        <v>14.74294533333333</v>
+        <v>12.56597571953333</v>
       </c>
     </row>
     <row r="48">
@@ -43969,12 +43969,12 @@
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam Bộ</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>Tây Ninh</t>
+          <t>Trà Vinh</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -43983,35 +43983,35 @@
         </is>
       </c>
       <c r="F48" s="37" t="n">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="G48" s="37" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H48" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I48" s="38" t="n">
-        <v>248</v>
+        <v>181</v>
       </c>
       <c r="J48" s="38" t="n">
-        <v>12.56597571953333</v>
+        <v>9.1493235976</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Đông Nam Bộ</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Trà Vinh</t>
+          <t>Đồng Nai</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
@@ -44020,35 +44020,35 @@
         </is>
       </c>
       <c r="F49" s="37" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="G49" s="37" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="H49" s="37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49" s="38" t="n">
-        <v>181</v>
+        <v>175.0833333333333</v>
       </c>
       <c r="J49" s="38" t="n">
-        <v>9.1493235976</v>
+        <v>8.503919416666667</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam Bộ</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Đồng Nai</t>
+          <t>Bắc Giang</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -44057,19 +44057,19 @@
         </is>
       </c>
       <c r="F50" s="37" t="n">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="G50" s="37" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H50" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I50" s="38" t="n">
-        <v>175.0833333333333</v>
+        <v>174</v>
       </c>
       <c r="J50" s="38" t="n">
-        <v>8.503919416666667</v>
+        <v>10.6188875</v>
       </c>
     </row>
     <row r="51">
@@ -44080,12 +44080,12 @@
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>Bắc Giang</t>
+          <t>Nghệ An</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
@@ -44094,19 +44094,19 @@
         </is>
       </c>
       <c r="F51" s="37" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G51" s="37" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H51" s="37" t="n">
         <v>3</v>
       </c>
       <c r="I51" s="38" t="n">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="J51" s="38" t="n">
-        <v>10.6188875</v>
+        <v>7.886790275833333</v>
       </c>
     </row>
     <row r="52">
@@ -44117,12 +44117,12 @@
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Nghệ An</t>
+          <t>Bạc Liêu</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -44131,7 +44131,7 @@
         </is>
       </c>
       <c r="F52" s="37" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G52" s="37" t="n">
         <v>11</v>
@@ -44140,10 +44140,10 @@
         <v>3</v>
       </c>
       <c r="I52" s="38" t="n">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J52" s="38" t="n">
-        <v>7.886790275833333</v>
+        <v>9.4811169056</v>
       </c>
     </row>
     <row r="53">
@@ -44159,7 +44159,7 @@
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Bạc Liêu</t>
+          <t>Sóc Trăng</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
@@ -44168,19 +44168,19 @@
         </is>
       </c>
       <c r="F53" s="37" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G53" s="37" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H53" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I53" s="38" t="n">
-        <v>165</v>
+        <v>126</v>
       </c>
       <c r="J53" s="38" t="n">
-        <v>9.4811169056</v>
+        <v>5.874500050666667</v>
       </c>
     </row>
     <row r="54">
@@ -44191,12 +44191,12 @@
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Sóc Trăng</t>
+          <t>Thái Nguyên</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -44205,35 +44205,35 @@
         </is>
       </c>
       <c r="F54" s="37" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="G54" s="37" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H54" s="37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I54" s="38" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J54" s="38" t="n">
-        <v>5.874500050666667</v>
+        <v>6.224007500000001</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>Thái Nguyên</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
@@ -44242,35 +44242,35 @@
         </is>
       </c>
       <c r="F55" s="37" t="n">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="G55" s="37" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H55" s="37" t="n">
         <v>3</v>
       </c>
       <c r="I55" s="38" t="n">
-        <v>122</v>
+        <v>105.4583333333333</v>
       </c>
       <c r="J55" s="38" t="n">
-        <v>6.224007500000001</v>
+        <v>6.507103091666667</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Hậu Giang</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -44279,19 +44279,19 @@
         </is>
       </c>
       <c r="F56" s="37" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H56" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I56" s="38" t="n">
-        <v>105.4583333333333</v>
+        <v>105</v>
       </c>
       <c r="J56" s="38" t="n">
-        <v>6.507103091666667</v>
+        <v>4.991647358333333</v>
       </c>
     </row>
     <row r="57">
@@ -44302,12 +44302,12 @@
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>Hậu Giang</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
@@ -44316,35 +44316,35 @@
         </is>
       </c>
       <c r="F57" s="37" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H57" s="37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I57" s="38" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="J57" s="38" t="n">
-        <v>4.991647358333333</v>
+        <v>6.821913375</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>An Giang</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -44353,35 +44353,35 @@
         </is>
       </c>
       <c r="F58" s="37" t="n">
-        <v>16</v>
+        <v>70</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="H58" s="37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I58" s="38" t="n">
-        <v>101</v>
+        <v>100.5</v>
       </c>
       <c r="J58" s="38" t="n">
-        <v>6.821913375</v>
+        <v>6.800787083333334</v>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>An Giang</t>
+          <t>Yên Bái</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
@@ -44390,19 +44390,19 @@
         </is>
       </c>
       <c r="F59" s="37" t="n">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="H59" s="37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I59" s="38" t="n">
-        <v>100.5</v>
+        <v>91</v>
       </c>
       <c r="J59" s="38" t="n">
-        <v>6.800787083333334</v>
+        <v>4.829244500000001</v>
       </c>
     </row>
     <row r="60">
@@ -44413,12 +44413,12 @@
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>Yên Bái</t>
+          <t>Nam Định</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
@@ -44427,19 +44427,19 @@
         </is>
       </c>
       <c r="F60" s="37" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H60" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I60" s="38" t="n">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="J60" s="38" t="n">
-        <v>4.829244500000001</v>
+        <v>4.559153395833333</v>
       </c>
     </row>
     <row r="61">
@@ -44455,7 +44455,7 @@
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Nam Định</t>
+          <t>Ninh Bình</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
@@ -44464,35 +44464,35 @@
         </is>
       </c>
       <c r="F61" s="37" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H61" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I61" s="38" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="J61" s="38" t="n">
-        <v>4.559153395833333</v>
+        <v>4.363913854166666</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Thanh Hóa</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -44501,35 +44501,35 @@
         </is>
       </c>
       <c r="F62" s="37" t="n">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="G62" s="37" t="n">
+        <v>21</v>
+      </c>
+      <c r="H62" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="H62" s="37" t="n">
-        <v>1</v>
-      </c>
       <c r="I62" s="38" t="n">
-        <v>69</v>
+        <v>68.25</v>
       </c>
       <c r="J62" s="38" t="n">
-        <v>4.363913854166666</v>
+        <v>5.044169338750001</v>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Tây Nguyên</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Thanh Hóa</t>
+          <t>Kon Tum</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
@@ -44538,19 +44538,19 @@
         </is>
       </c>
       <c r="F63" s="37" t="n">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="H63" s="37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I63" s="38" t="n">
-        <v>68.25</v>
+        <v>65</v>
       </c>
       <c r="J63" s="38" t="n">
-        <v>5.044169338750001</v>
+        <v>3.922742576</v>
       </c>
     </row>
     <row r="64">
@@ -44566,7 +44566,7 @@
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>Kon Tum</t>
+          <t>Đắk Nông</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
@@ -44575,19 +44575,19 @@
         </is>
       </c>
       <c r="F64" s="37" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H64" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="38" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J64" s="38" t="n">
-        <v>3.922742576</v>
+        <v>3.474977075333333</v>
       </c>
     </row>
     <row r="65">
@@ -44598,12 +44598,12 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Tây Nguyên</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Đắk Nông</t>
+          <t>Hưng Yên</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
@@ -44612,19 +44612,19 @@
         </is>
       </c>
       <c r="F65" s="37" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="G65" s="37" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H65" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I65" s="38" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J65" s="38" t="n">
-        <v>3.474977075333333</v>
+        <v>4.636627</v>
       </c>
     </row>
     <row r="66">
@@ -44640,7 +44640,7 @@
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>Hưng Yên</t>
+          <t>Vĩnh Phúc</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -44649,35 +44649,35 @@
         </is>
       </c>
       <c r="F66" s="37" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G66" s="37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H66" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I66" s="38" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="J66" s="38" t="n">
-        <v>4.636627</v>
+        <v>2.544545</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Vĩnh Phúc</t>
+          <t>Huế</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
@@ -44686,7 +44686,7 @@
         </is>
       </c>
       <c r="F67" s="37" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="G67" s="37" t="n">
         <v>5</v>
@@ -44695,10 +44695,10 @@
         <v>2</v>
       </c>
       <c r="I67" s="38" t="n">
-        <v>52</v>
+        <v>48.5</v>
       </c>
       <c r="J67" s="38" t="n">
-        <v>2.544545</v>
+        <v>2.4148221875</v>
       </c>
     </row>
     <row r="68">
@@ -44714,7 +44714,7 @@
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>Huế</t>
+          <t>Quảng Ngãi</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
@@ -44723,19 +44723,19 @@
         </is>
       </c>
       <c r="F68" s="37" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="G68" s="37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H68" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I68" s="38" t="n">
-        <v>48.5</v>
+        <v>45.16666666666666</v>
       </c>
       <c r="J68" s="38" t="n">
-        <v>2.4148221875</v>
+        <v>6.77718966</v>
       </c>
     </row>
     <row r="69">
@@ -44746,12 +44746,12 @@
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>Quảng Ngãi</t>
+          <t>Phú Thọ</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
@@ -44760,25 +44760,25 @@
         </is>
       </c>
       <c r="F69" s="37" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H69" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I69" s="38" t="n">
-        <v>45.16666666666666</v>
+        <v>34.08333333333334</v>
       </c>
       <c r="J69" s="38" t="n">
-        <v>6.77718966</v>
+        <v>1.775710916666667</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C70" s="12" t="inlineStr">
@@ -44788,7 +44788,7 @@
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Phú Thọ</t>
+          <t>Tuyên Quang</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
@@ -44797,19 +44797,19 @@
         </is>
       </c>
       <c r="F70" s="37" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H70" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I70" s="38" t="n">
-        <v>34.08333333333334</v>
+        <v>31</v>
       </c>
       <c r="J70" s="38" t="n">
-        <v>1.775710916666667</v>
+        <v>2.154967</v>
       </c>
     </row>
     <row r="71">
@@ -44820,12 +44820,12 @@
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Tuyên Quang</t>
+          <t>Hà Tĩnh</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
@@ -44834,25 +44834,25 @@
         </is>
       </c>
       <c r="F71" s="37" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H71" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I71" s="38" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J71" s="38" t="n">
-        <v>2.154967</v>
+        <v>1.797568833333334</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C72" s="12" t="inlineStr">
@@ -44862,7 +44862,7 @@
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Hà Tĩnh</t>
+          <t>Nghệ An</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
@@ -44871,35 +44871,35 @@
         </is>
       </c>
       <c r="F72" s="37" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H72" s="37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I72" s="38" t="n">
-        <v>30</v>
+        <v>28.91666666666667</v>
       </c>
       <c r="J72" s="38" t="n">
-        <v>1.797568833333334</v>
+        <v>1.893862708333333</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Nghệ An</t>
+          <t>Hà Giang</t>
         </is>
       </c>
       <c r="E73" s="12" t="inlineStr">
@@ -44908,35 +44908,35 @@
         </is>
       </c>
       <c r="F73" s="37" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H73" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I73" s="38" t="n">
-        <v>28.91666666666667</v>
+        <v>26</v>
       </c>
       <c r="J73" s="38" t="n">
-        <v>1.893862708333333</v>
+        <v>1.938676833333333</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Tây Nguyên</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Hà Giang</t>
+          <t>Gia Lai</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
@@ -44945,19 +44945,19 @@
         </is>
       </c>
       <c r="F74" s="37" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H74" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I74" s="38" t="n">
-        <v>26</v>
+        <v>25.41666666666667</v>
       </c>
       <c r="J74" s="38" t="n">
-        <v>1.938676833333333</v>
+        <v>3.474808159666667</v>
       </c>
     </row>
     <row r="75">
@@ -44968,12 +44968,12 @@
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>Tây Nguyên</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>Gia Lai</t>
+          <t>Kiên Giang</t>
         </is>
       </c>
       <c r="E75" s="12" t="inlineStr">
@@ -44982,35 +44982,35 @@
         </is>
       </c>
       <c r="F75" s="37" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H75" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I75" s="38" t="n">
-        <v>25.41666666666667</v>
+        <v>25.41666666666666</v>
       </c>
       <c r="J75" s="38" t="n">
-        <v>3.474808159666667</v>
+        <v>1.94346388325</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Kiên Giang</t>
+          <t>Lào Cai</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -45019,7 +45019,7 @@
         </is>
       </c>
       <c r="F76" s="37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G76" s="37" t="n">
         <v>4</v>
@@ -45028,26 +45028,26 @@
         <v>1</v>
       </c>
       <c r="I76" s="38" t="n">
-        <v>25.41666666666666</v>
+        <v>25</v>
       </c>
       <c r="J76" s="38" t="n">
-        <v>1.94346388325</v>
+        <v>1.523068375</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>Lào Cai</t>
+          <t>Nam Định</t>
         </is>
       </c>
       <c r="E77" s="12" t="inlineStr">
@@ -45056,35 +45056,35 @@
         </is>
       </c>
       <c r="F77" s="37" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H77" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I77" s="38" t="n">
-        <v>25</v>
+        <v>20.41666666666667</v>
       </c>
       <c r="J77" s="38" t="n">
-        <v>1.523068375</v>
+        <v>1.55470140375</v>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Nam Định</t>
+          <t>Sơn La</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
@@ -45093,19 +45093,19 @@
         </is>
       </c>
       <c r="F78" s="37" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H78" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78" s="38" t="n">
-        <v>20.41666666666667</v>
+        <v>20</v>
       </c>
       <c r="J78" s="38" t="n">
-        <v>1.55470140375</v>
+        <v>1.15875</v>
       </c>
     </row>
     <row r="79">
@@ -45116,12 +45116,12 @@
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>Sơn La</t>
+          <t>Thái Bình</t>
         </is>
       </c>
       <c r="E79" s="12" t="inlineStr">
@@ -45130,10 +45130,10 @@
         </is>
       </c>
       <c r="F79" s="37" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G79" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H79" s="37" t="n">
         <v>1</v>
@@ -45142,7 +45142,7 @@
         <v>20</v>
       </c>
       <c r="J79" s="38" t="n">
-        <v>1.15875</v>
+        <v>1.2304015</v>
       </c>
     </row>
     <row r="80">
@@ -45153,12 +45153,12 @@
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Thái Bình</t>
+          <t>Lạng Sơn</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
@@ -45167,19 +45167,19 @@
         </is>
       </c>
       <c r="F80" s="37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G80" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H80" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I80" s="38" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J80" s="38" t="n">
-        <v>1.2304015</v>
+        <v>1.09726</v>
       </c>
     </row>
     <row r="81">
@@ -45195,7 +45195,7 @@
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>Lạng Sơn</t>
+          <t>Hòa Bình</t>
         </is>
       </c>
       <c r="E81" s="12" t="inlineStr">
@@ -45204,35 +45204,35 @@
         </is>
       </c>
       <c r="F81" s="37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G81" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H81" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I81" s="38" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J81" s="38" t="n">
-        <v>1.09726</v>
+        <v>1.263885</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Hòa Bình</t>
+          <t>Quảng Nam</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
@@ -45241,19 +45241,19 @@
         </is>
       </c>
       <c r="F82" s="37" t="n">
+        <v>12</v>
+      </c>
+      <c r="G82" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="G82" s="37" t="n">
+      <c r="H82" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="H82" s="37" t="n">
-        <v>1</v>
-      </c>
       <c r="I82" s="38" t="n">
-        <v>16</v>
+        <v>14.75</v>
       </c>
       <c r="J82" s="38" t="n">
-        <v>1.263885</v>
+        <v>1.411311541666667</v>
       </c>
     </row>
     <row r="83">
@@ -45264,12 +45264,12 @@
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>Quảng Nam</t>
+          <t>Quảng Ninh</t>
         </is>
       </c>
       <c r="E83" s="12" t="inlineStr">
@@ -45278,19 +45278,19 @@
         </is>
       </c>
       <c r="F83" s="37" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G83" s="37" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H83" s="37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I83" s="38" t="n">
-        <v>14.75</v>
+        <v>13.91666666666667</v>
       </c>
       <c r="J83" s="38" t="n">
-        <v>1.411311541666667</v>
+        <v>0.7997978958333334</v>
       </c>
     </row>
     <row r="84">
@@ -45301,12 +45301,12 @@
       </c>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Hải Dương</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
@@ -45315,19 +45315,19 @@
         </is>
       </c>
       <c r="F84" s="37" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G84" s="37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H84" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I84" s="38" t="n">
-        <v>13.91666666666667</v>
+        <v>13.83333333333333</v>
       </c>
       <c r="J84" s="38" t="n">
-        <v>0.7997978958333334</v>
+        <v>1.069398479166667</v>
       </c>
     </row>
     <row r="85">
@@ -45338,12 +45338,12 @@
       </c>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>Hải Dương</t>
+          <t>Quảng Bình</t>
         </is>
       </c>
       <c r="E85" s="12" t="inlineStr">
@@ -45352,19 +45352,19 @@
         </is>
       </c>
       <c r="F85" s="37" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G85" s="37" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H85" s="37" t="n">
         <v>2</v>
       </c>
       <c r="I85" s="38" t="n">
-        <v>13.83333333333333</v>
+        <v>12.83333333333333</v>
       </c>
       <c r="J85" s="38" t="n">
-        <v>1.069398479166667</v>
+        <v>1.130885083333333</v>
       </c>
     </row>
     <row r="86">
@@ -45375,12 +45375,12 @@
       </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đông Nam Bộ</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Quảng Bình</t>
+          <t>Bình Phước</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
@@ -45389,19 +45389,19 @@
         </is>
       </c>
       <c r="F86" s="37" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G86" s="37" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H86" s="37" t="n">
         <v>2</v>
       </c>
       <c r="I86" s="38" t="n">
-        <v>12.83333333333333</v>
+        <v>12.75</v>
       </c>
       <c r="J86" s="38" t="n">
-        <v>1.130885083333333</v>
+        <v>0.8002302083333334</v>
       </c>
     </row>
     <row r="87">
@@ -45412,12 +45412,12 @@
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam Bộ</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
-          <t>Bình Phước</t>
+          <t>Yên Bái</t>
         </is>
       </c>
       <c r="E87" s="12" t="inlineStr">
@@ -45426,19 +45426,19 @@
         </is>
       </c>
       <c r="F87" s="37" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G87" s="37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H87" s="37" t="n">
         <v>2</v>
       </c>
       <c r="I87" s="38" t="n">
-        <v>12.75</v>
+        <v>12.08333333333333</v>
       </c>
       <c r="J87" s="38" t="n">
-        <v>0.8002302083333334</v>
+        <v>0.9781446875000001</v>
       </c>
     </row>
     <row r="88">
@@ -45454,7 +45454,7 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Yên Bái</t>
+          <t>Thái Nguyên</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
@@ -45463,19 +45463,19 @@
         </is>
       </c>
       <c r="F88" s="37" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G88" s="37" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H88" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I88" s="38" t="n">
-        <v>12.08333333333333</v>
+        <v>12</v>
       </c>
       <c r="J88" s="38" t="n">
-        <v>0.9781446875000001</v>
+        <v>0.8894690541666668</v>
       </c>
     </row>
     <row r="89">
@@ -45486,12 +45486,12 @@
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D89" s="12" t="inlineStr">
         <is>
-          <t>Thái Nguyên</t>
+          <t>Ninh Bình</t>
         </is>
       </c>
       <c r="E89" s="12" t="inlineStr">
@@ -45500,19 +45500,19 @@
         </is>
       </c>
       <c r="F89" s="37" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G89" s="37" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H89" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I89" s="38" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J89" s="38" t="n">
-        <v>0.8894690541666668</v>
+        <v>0.6863781250000001</v>
       </c>
     </row>
     <row r="90">
@@ -45528,7 +45528,7 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Vĩnh Phúc</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -45537,19 +45537,19 @@
         </is>
       </c>
       <c r="F90" s="37" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G90" s="37" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H90" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I90" s="38" t="n">
-        <v>11</v>
+        <v>10.83333333333333</v>
       </c>
       <c r="J90" s="38" t="n">
-        <v>0.6863781250000001</v>
+        <v>0.6501950625</v>
       </c>
     </row>
     <row r="91">
@@ -45560,12 +45560,12 @@
       </c>
       <c r="C91" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D91" s="12" t="inlineStr">
         <is>
-          <t>Vĩnh Phúc</t>
+          <t>Phú Yên</t>
         </is>
       </c>
       <c r="E91" s="12" t="inlineStr">
@@ -45574,19 +45574,19 @@
         </is>
       </c>
       <c r="F91" s="37" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G91" s="37" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H91" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I91" s="38" t="n">
-        <v>10.83333333333333</v>
+        <v>10.33333333333333</v>
       </c>
       <c r="J91" s="38" t="n">
-        <v>0.6501950625</v>
+        <v>1.013268354166667</v>
       </c>
     </row>
     <row r="92">
@@ -45597,12 +45597,12 @@
       </c>
       <c r="C92" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Phú Yên</t>
+          <t>Vĩnh Long</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
@@ -45611,19 +45611,19 @@
         </is>
       </c>
       <c r="F92" s="37" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G92" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H92" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I92" s="38" t="n">
-        <v>10.33333333333333</v>
+        <v>9.75</v>
       </c>
       <c r="J92" s="38" t="n">
-        <v>1.013268354166667</v>
+        <v>0.7372540833333334</v>
       </c>
     </row>
     <row r="93">
@@ -45634,12 +45634,12 @@
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr">
         <is>
-          <t>Vĩnh Long</t>
+          <t>Hà Tĩnh</t>
         </is>
       </c>
       <c r="E93" s="12" t="inlineStr">
@@ -45648,35 +45648,35 @@
         </is>
       </c>
       <c r="F93" s="37" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G93" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H93" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="H93" s="37" t="n">
-        <v>1</v>
-      </c>
       <c r="I93" s="38" t="n">
-        <v>9.75</v>
+        <v>9.5</v>
       </c>
       <c r="J93" s="38" t="n">
-        <v>0.7372540833333334</v>
+        <v>0.9184344166666667</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>Vinh Loc</t>
+          <t>My Phuoc</t>
         </is>
       </c>
       <c r="C94" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Hà Tĩnh</t>
+          <t>Hà Nam</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
@@ -45685,25 +45685,25 @@
         </is>
       </c>
       <c r="F94" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G94" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H94" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I94" s="38" t="n">
         <v>9</v>
       </c>
-      <c r="G94" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="H94" s="37" t="n">
-        <v>2</v>
-      </c>
-      <c r="I94" s="38" t="n">
-        <v>9.5</v>
-      </c>
       <c r="J94" s="38" t="n">
-        <v>0.9184344166666667</v>
+        <v>0.6445000000000001</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="12" t="inlineStr">
         <is>
-          <t>My Phuoc</t>
+          <t>Vinh Loc</t>
         </is>
       </c>
       <c r="C95" s="12" t="inlineStr">
@@ -45713,7 +45713,7 @@
       </c>
       <c r="D95" s="12" t="inlineStr">
         <is>
-          <t>Hà Nam</t>
+          <t>Hưng Yên</t>
         </is>
       </c>
       <c r="E95" s="12" t="inlineStr">
@@ -45722,19 +45722,19 @@
         </is>
       </c>
       <c r="F95" s="37" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G95" s="37" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H95" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I95" s="38" t="n">
-        <v>9</v>
+        <v>8.916666666666666</v>
       </c>
       <c r="J95" s="38" t="n">
-        <v>0.6445000000000001</v>
+        <v>0.63316775</v>
       </c>
     </row>
     <row r="96">
@@ -45745,12 +45745,12 @@
       </c>
       <c r="C96" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Hưng Yên</t>
+          <t>Bến Tre</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
@@ -45759,19 +45759,19 @@
         </is>
       </c>
       <c r="F96" s="37" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G96" s="37" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H96" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I96" s="38" t="n">
-        <v>8.916666666666666</v>
+        <v>8.833333333333334</v>
       </c>
       <c r="J96" s="38" t="n">
-        <v>0.63316775</v>
+        <v>1.087301333333333</v>
       </c>
     </row>
     <row r="97">
@@ -45782,12 +45782,12 @@
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Tây Nguyên</t>
         </is>
       </c>
       <c r="D97" s="12" t="inlineStr">
         <is>
-          <t>Bến Tre</t>
+          <t>Lâm Đồng</t>
         </is>
       </c>
       <c r="E97" s="12" t="inlineStr">
@@ -45796,19 +45796,19 @@
         </is>
       </c>
       <c r="F97" s="37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G97" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H97" s="37" t="n">
         <v>2</v>
       </c>
       <c r="I97" s="38" t="n">
-        <v>8.833333333333334</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="J97" s="38" t="n">
-        <v>1.087301333333333</v>
+        <v>0.8673489083333333</v>
       </c>
     </row>
     <row r="98">
@@ -45819,12 +45819,12 @@
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>Tây Nguyên</t>
+          <t>Đồng bằng sông Hồng</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Lâm Đồng</t>
+          <t>Thái Bình</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
@@ -45833,19 +45833,19 @@
         </is>
       </c>
       <c r="F98" s="37" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G98" s="37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H98" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I98" s="38" t="n">
-        <v>8.333333333333334</v>
+        <v>7.083333333333333</v>
       </c>
       <c r="J98" s="38" t="n">
-        <v>0.8673489083333333</v>
+        <v>0.4130432708333334</v>
       </c>
     </row>
     <row r="99">
@@ -45861,7 +45861,7 @@
       </c>
       <c r="D99" s="12" t="inlineStr">
         <is>
-          <t>Thái Bình</t>
+          <t>Hà Nam</t>
         </is>
       </c>
       <c r="E99" s="12" t="inlineStr">
@@ -45870,19 +45870,19 @@
         </is>
       </c>
       <c r="F99" s="37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G99" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H99" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I99" s="38" t="n">
-        <v>7.083333333333333</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="J99" s="38" t="n">
-        <v>0.4130432708333334</v>
+        <v>0.436776125</v>
       </c>
     </row>
     <row r="100">
@@ -45893,12 +45893,12 @@
       </c>
       <c r="C100" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Hồng</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Hà Nam</t>
+          <t>Hậu Giang</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
@@ -45907,19 +45907,19 @@
         </is>
       </c>
       <c r="F100" s="37" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G100" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H100" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I100" s="38" t="n">
-        <v>6.666666666666667</v>
+        <v>6.333333333333334</v>
       </c>
       <c r="J100" s="38" t="n">
-        <v>0.436776125</v>
+        <v>0.6552413333333333</v>
       </c>
     </row>
     <row r="101">
@@ -45935,7 +45935,7 @@
       </c>
       <c r="D101" s="12" t="inlineStr">
         <is>
-          <t>Hậu Giang</t>
+          <t>Bạc Liêu</t>
         </is>
       </c>
       <c r="E101" s="12" t="inlineStr">
@@ -45953,10 +45953,10 @@
         <v>1</v>
       </c>
       <c r="I101" s="38" t="n">
-        <v>6.333333333333334</v>
+        <v>6</v>
       </c>
       <c r="J101" s="38" t="n">
-        <v>0.6552413333333333</v>
+        <v>0.6317440000000001</v>
       </c>
     </row>
     <row r="102">
@@ -45972,7 +45972,7 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Bạc Liêu</t>
+          <t>Trà Vinh</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
@@ -45981,10 +45981,10 @@
         </is>
       </c>
       <c r="F102" s="37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G102" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H102" s="37" t="n">
         <v>1</v>
@@ -45993,7 +45993,7 @@
         <v>6</v>
       </c>
       <c r="J102" s="38" t="n">
-        <v>0.6317440000000001</v>
+        <v>0.9877725900000001</v>
       </c>
     </row>
     <row r="103">
@@ -46004,12 +46004,12 @@
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D103" s="12" t="inlineStr">
         <is>
-          <t>Trà Vinh</t>
+          <t>Điện Biên</t>
         </is>
       </c>
       <c r="E103" s="12" t="inlineStr">
@@ -46018,19 +46018,19 @@
         </is>
       </c>
       <c r="F103" s="37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G103" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H103" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I103" s="38" t="n">
-        <v>6</v>
+        <v>5.833333333333334</v>
       </c>
       <c r="J103" s="38" t="n">
-        <v>0.9877725900000001</v>
+        <v>0.5906513333333333</v>
       </c>
     </row>
     <row r="104">
@@ -46041,12 +46041,12 @@
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Điện Biên</t>
+          <t>Long An</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
@@ -46064,10 +46064,10 @@
         <v>1</v>
       </c>
       <c r="I104" s="38" t="n">
-        <v>5.833333333333334</v>
+        <v>5.5</v>
       </c>
       <c r="J104" s="38" t="n">
-        <v>0.5906513333333333</v>
+        <v>0.573222</v>
       </c>
     </row>
     <row r="105">
@@ -46078,12 +46078,12 @@
       </c>
       <c r="C105" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
         </is>
       </c>
       <c r="D105" s="12" t="inlineStr">
         <is>
-          <t>Long An</t>
+          <t>Bình Định</t>
         </is>
       </c>
       <c r="E105" s="12" t="inlineStr">
@@ -46101,10 +46101,10 @@
         <v>1</v>
       </c>
       <c r="I105" s="38" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="J105" s="38" t="n">
-        <v>0.573222</v>
+        <v>0.497982</v>
       </c>
     </row>
     <row r="106">
@@ -46115,12 +46115,12 @@
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>Bắc Trung Bộ và Duyên hải miền Trung</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Bình Định</t>
+          <t>Lạng Sơn</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
@@ -46129,19 +46129,19 @@
         </is>
       </c>
       <c r="F106" s="37" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G106" s="37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H106" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I106" s="38" t="n">
-        <v>5</v>
+        <v>4.791666666666666</v>
       </c>
       <c r="J106" s="38" t="n">
-        <v>0.497982</v>
+        <v>0.367813125</v>
       </c>
     </row>
     <row r="107">
@@ -46157,7 +46157,7 @@
       </c>
       <c r="D107" s="12" t="inlineStr">
         <is>
-          <t>Lạng Sơn</t>
+          <t>Bắc Kạn</t>
         </is>
       </c>
       <c r="E107" s="12" t="inlineStr">
@@ -46166,7 +46166,7 @@
         </is>
       </c>
       <c r="F107" s="37" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G107" s="37" t="n">
         <v>5</v>
@@ -46175,10 +46175,10 @@
         <v>1</v>
       </c>
       <c r="I107" s="38" t="n">
-        <v>4.791666666666666</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="J107" s="38" t="n">
-        <v>0.367813125</v>
+        <v>0.2954270000000001</v>
       </c>
     </row>
     <row r="108">
@@ -46194,7 +46194,7 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Bắc Kạn</t>
+          <t>Hòa Bình</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
@@ -46206,7 +46206,7 @@
         <v>5</v>
       </c>
       <c r="G108" s="37" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H108" s="37" t="n">
         <v>1</v>
@@ -46215,7 +46215,7 @@
         <v>4.666666666666667</v>
       </c>
       <c r="J108" s="38" t="n">
-        <v>0.2954270000000001</v>
+        <v>0.2939400625</v>
       </c>
     </row>
     <row r="109">
@@ -46231,7 +46231,7 @@
       </c>
       <c r="D109" s="12" t="inlineStr">
         <is>
-          <t>Hòa Bình</t>
+          <t>Hà Giang</t>
         </is>
       </c>
       <c r="E109" s="12" t="inlineStr">
@@ -46240,19 +46240,19 @@
         </is>
       </c>
       <c r="F109" s="37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G109" s="37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H109" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I109" s="38" t="n">
-        <v>4.666666666666667</v>
+        <v>3.25</v>
       </c>
       <c r="J109" s="38" t="n">
-        <v>0.2939400625</v>
+        <v>0.23787675</v>
       </c>
     </row>
     <row r="110">
@@ -46263,12 +46263,12 @@
       </c>
       <c r="C110" s="12" t="inlineStr">
         <is>
-          <t>Trung du và miền núi phía Bắc</t>
+          <t>Đồng bằng sông Cửu Long</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Hà Giang</t>
+          <t>Cà Mau</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
@@ -46277,19 +46277,19 @@
         </is>
       </c>
       <c r="F110" s="37" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G110" s="37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H110" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I110" s="38" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="J110" s="38" t="n">
-        <v>0.23787675</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="111">
@@ -46300,12 +46300,12 @@
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>Đồng bằng sông Cửu Long</t>
+          <t>Trung du và miền núi phía Bắc</t>
         </is>
       </c>
       <c r="D111" s="12" t="inlineStr">
         <is>
-          <t>Cà Mau</t>
+          <t>Bắc Giang</t>
         </is>
       </c>
       <c r="E111" s="12" t="inlineStr">
@@ -46314,7 +46314,7 @@
         </is>
       </c>
       <c r="F111" s="37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G111" s="37" t="n">
         <v>2</v>
@@ -46323,10 +46323,10 @@
         <v>1</v>
       </c>
       <c r="I111" s="38" t="n">
-        <v>3</v>
+        <v>2.833333333333333</v>
       </c>
       <c r="J111" s="38" t="n">
-        <v>0.486</v>
+        <v>0.168922</v>
       </c>
     </row>
     <row r="112">
@@ -46342,7 +46342,7 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Bắc Giang</t>
+          <t>Lào Cai</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
@@ -46351,60 +46351,23 @@
         </is>
       </c>
       <c r="F112" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G112" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H112" s="37" t="n">
         <v>1</v>
       </c>
       <c r="I112" s="38" t="n">
-        <v>2.833333333333333</v>
+        <v>2.166666666666667</v>
       </c>
       <c r="J112" s="38" t="n">
-        <v>0.168922</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="B113" s="12" t="inlineStr">
-        <is>
-          <t>Vinh Loc</t>
-        </is>
-      </c>
-      <c r="C113" s="12" t="inlineStr">
-        <is>
-          <t>Trung du và miền núi phía Bắc</t>
-        </is>
-      </c>
-      <c r="D113" s="12" t="inlineStr">
-        <is>
-          <t>Lào Cai</t>
-        </is>
-      </c>
-      <c r="E113" s="12" t="inlineStr">
-        <is>
-          <t>distributor_match</t>
-        </is>
-      </c>
-      <c r="F113" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="G113" s="37" t="n">
-        <v>1</v>
-      </c>
-      <c r="H113" s="37" t="n">
-        <v>1</v>
-      </c>
-      <c r="I113" s="38" t="n">
-        <v>2.166666666666667</v>
-      </c>
-      <c r="J113" s="38" t="n">
         <v>0.108342</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:J113"/>
+  <autoFilter ref="B2:J112"/>
   <mergeCells count="1">
     <mergeCell ref="B1:J1"/>
   </mergeCells>
@@ -46418,7 +46381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P17"/>
+  <dimension ref="B1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -46628,41 +46591,41 @@
     <row r="5">
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Đồng Nai</t>
+          <t>Đà Nẵng</t>
         </is>
       </c>
       <c r="C5" s="37" t="n">
-        <v>1356</v>
+        <v>1317</v>
       </c>
       <c r="D5" s="37" t="n">
-        <v>434</v>
+        <v>296</v>
       </c>
       <c r="E5" s="37" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="38" t="n">
-        <v>6080.083333333333</v>
+        <v>24340.47916666667</v>
       </c>
       <c r="G5" s="38" t="n">
-        <v>283.9447239694703</v>
+        <v>1460.204066025033</v>
       </c>
       <c r="H5" s="37" t="n">
-        <v>409</v>
+        <v>230</v>
       </c>
       <c r="I5" s="37" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="J5" s="38" t="n">
-        <v>5905</v>
+        <v>23428</v>
       </c>
       <c r="K5" s="38" t="n">
-        <v>175.0833333333333</v>
+        <v>912.4791666666666</v>
       </c>
       <c r="L5" s="38" t="n">
-        <v>0.9712037938076508</v>
+        <v>0.9625118650944114</v>
       </c>
       <c r="M5" s="38" t="n">
-        <v>0.02879620619234934</v>
+        <v>0.03748813490558851</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
@@ -46673,47 +46636,47 @@
         <v>3</v>
       </c>
       <c r="P5" s="37" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Đà Nẵng</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="C6" s="37" t="n">
-        <v>1317</v>
+        <v>837</v>
       </c>
       <c r="D6" s="37" t="n">
-        <v>296</v>
+        <v>280</v>
       </c>
       <c r="E6" s="37" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F6" s="38" t="n">
-        <v>24340.47916666667</v>
+        <v>13142.66666666667</v>
       </c>
       <c r="G6" s="38" t="n">
-        <v>1460.204066025033</v>
+        <v>822.4895296015001</v>
       </c>
       <c r="H6" s="37" t="n">
-        <v>230</v>
+        <v>145</v>
       </c>
       <c r="I6" s="37" t="n">
-        <v>66</v>
+        <v>135</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>23428</v>
+        <v>10950</v>
       </c>
       <c r="K6" s="38" t="n">
-        <v>912.4791666666666</v>
+        <v>2192.666666666667</v>
       </c>
       <c r="L6" s="38" t="n">
-        <v>0.9625118650944114</v>
+        <v>0.8331642487572284</v>
       </c>
       <c r="M6" s="38" t="n">
-        <v>0.03748813490558851</v>
+        <v>0.1668357512427716</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
@@ -46724,47 +46687,47 @@
         <v>4</v>
       </c>
       <c r="P6" s="37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hà Nội</t>
+          <t>Cần Thơ</t>
         </is>
       </c>
       <c r="C7" s="37" t="n">
-        <v>837</v>
+        <v>1094</v>
       </c>
       <c r="D7" s="37" t="n">
-        <v>280</v>
+        <v>257</v>
       </c>
       <c r="E7" s="37" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F7" s="38" t="n">
-        <v>13142.66666666667</v>
+        <v>19444.875</v>
       </c>
       <c r="G7" s="38" t="n">
-        <v>822.4895296015001</v>
+        <v>1162.38288698675</v>
       </c>
       <c r="H7" s="37" t="n">
-        <v>145</v>
+        <v>207</v>
       </c>
       <c r="I7" s="37" t="n">
-        <v>135</v>
+        <v>50</v>
       </c>
       <c r="J7" s="38" t="n">
-        <v>10950</v>
+        <v>18676</v>
       </c>
       <c r="K7" s="38" t="n">
-        <v>2192.666666666667</v>
+        <v>768.875</v>
       </c>
       <c r="L7" s="38" t="n">
-        <v>0.8331642487572284</v>
+        <v>0.9604587326994902</v>
       </c>
       <c r="M7" s="38" t="n">
-        <v>0.1668357512427716</v>
+        <v>0.03954126730050977</v>
       </c>
       <c r="N7" s="12" t="inlineStr">
         <is>
@@ -46775,47 +46738,47 @@
         <v>5</v>
       </c>
       <c r="P7" s="37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Cần Thơ</t>
+          <t>Khánh Hòa</t>
         </is>
       </c>
       <c r="C8" s="37" t="n">
-        <v>1094</v>
+        <v>839</v>
       </c>
       <c r="D8" s="37" t="n">
-        <v>257</v>
+        <v>200</v>
       </c>
       <c r="E8" s="37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" s="38" t="n">
-        <v>19444.875</v>
+        <v>12101.5</v>
       </c>
       <c r="G8" s="38" t="n">
-        <v>1162.38288698675</v>
+        <v>733.6744502710001</v>
       </c>
       <c r="H8" s="37" t="n">
-        <v>207</v>
+        <v>157</v>
       </c>
       <c r="I8" s="37" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="J8" s="38" t="n">
-        <v>18676</v>
+        <v>11644</v>
       </c>
       <c r="K8" s="38" t="n">
-        <v>768.875</v>
+        <v>457.5</v>
       </c>
       <c r="L8" s="38" t="n">
-        <v>0.9604587326994902</v>
+        <v>0.9621947692434822</v>
       </c>
       <c r="M8" s="38" t="n">
-        <v>0.03954126730050977</v>
+        <v>0.03780523075651779</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
@@ -46826,47 +46789,47 @@
         <v>6</v>
       </c>
       <c r="P8" s="37" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Khánh Hòa</t>
+          <t>Tiền Giang</t>
         </is>
       </c>
       <c r="C9" s="37" t="n">
-        <v>839</v>
+        <v>494</v>
       </c>
       <c r="D9" s="37" t="n">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="E9" s="37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" s="38" t="n">
-        <v>12101.5</v>
+        <v>12380.58333333333</v>
       </c>
       <c r="G9" s="38" t="n">
-        <v>733.6744502710001</v>
+        <v>774.4612576916667</v>
       </c>
       <c r="H9" s="37" t="n">
-        <v>157</v>
+        <v>124</v>
       </c>
       <c r="I9" s="37" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>11644</v>
+        <v>11673</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>457.5</v>
+        <v>707.5833333333334</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>0.9621947692434822</v>
+        <v>0.9428473348724817</v>
       </c>
       <c r="M9" s="38" t="n">
-        <v>0.03780523075651779</v>
+        <v>0.05715266512751822</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
@@ -46877,47 +46840,47 @@
         <v>7</v>
       </c>
       <c r="P9" s="37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Tiền Giang</t>
+          <t>Đồng Nai</t>
         </is>
       </c>
       <c r="C10" s="37" t="n">
-        <v>494</v>
+        <v>765</v>
       </c>
       <c r="D10" s="37" t="n">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="E10" s="37" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F10" s="38" t="n">
-        <v>12380.58333333333</v>
+        <v>4195.083333333333</v>
       </c>
       <c r="G10" s="38" t="n">
-        <v>774.4612576916667</v>
+        <v>193.8974272953334</v>
       </c>
       <c r="H10" s="37" t="n">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="I10" s="37" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="J10" s="38" t="n">
-        <v>11673</v>
+        <v>4020</v>
       </c>
       <c r="K10" s="38" t="n">
-        <v>707.5833333333334</v>
+        <v>175.0833333333333</v>
       </c>
       <c r="L10" s="38" t="n">
-        <v>0.9428473348724817</v>
+        <v>0.9582646351880177</v>
       </c>
       <c r="M10" s="38" t="n">
-        <v>0.05715266512751822</v>
+        <v>0.04173536481198228</v>
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
@@ -46928,7 +46891,7 @@
         <v>8</v>
       </c>
       <c r="P10" s="37" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -47030,7 +46993,7 @@
         <v>10</v>
       </c>
       <c r="P12" s="37" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -47183,7 +47146,7 @@
         <v>13</v>
       </c>
       <c r="P15" s="37" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -47234,7 +47197,7 @@
         <v>14</v>
       </c>
       <c r="P16" s="37" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -47285,11 +47248,62 @@
         <v>16</v>
       </c>
       <c r="P17" s="37" t="n">
-        <v>10</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Huế</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="n">
+        <v>271</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <v>62</v>
+      </c>
+      <c r="E18" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="38" t="n">
+        <v>4613.5</v>
+      </c>
+      <c r="G18" s="38" t="n">
+        <v>259.8426835653667</v>
+      </c>
+      <c r="H18" s="37" t="n">
+        <v>57</v>
+      </c>
+      <c r="I18" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" s="38" t="n">
+        <v>4565</v>
+      </c>
+      <c r="K18" s="38" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="L18" s="38" t="n">
+        <v>0.9894873740110545</v>
+      </c>
+      <c r="M18" s="38" t="n">
+        <v>0.01051262598894549</v>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>My Phuoc</t>
+        </is>
+      </c>
+      <c r="O18" s="37" t="n">
+        <v>17</v>
+      </c>
+      <c r="P18" s="37" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:P17"/>
+  <autoFilter ref="B2:P18"/>
   <mergeCells count="1">
     <mergeCell ref="B1:P1"/>
   </mergeCells>
@@ -47417,10 +47431,10 @@
         <v>0.9761378620498172</v>
       </c>
       <c r="K3" s="38" t="n">
-        <v>0.2283140283140283</v>
+        <v>0.2458425720620843</v>
       </c>
       <c r="L3" s="38" t="n">
-        <v>0.2666965721814052</v>
+        <v>0.2687438151823783</v>
       </c>
     </row>
     <row r="4">
@@ -47495,10 +47509,10 @@
         <v>0.9686617105211766</v>
       </c>
       <c r="K5" s="38" t="n">
-        <v>0.0241956241956242</v>
+        <v>0.02605321507760532</v>
       </c>
       <c r="L5" s="38" t="n">
-        <v>0.01252798590399522</v>
+        <v>0.01262415448707246</v>
       </c>
     </row>
     <row r="6">
@@ -47573,10 +47587,10 @@
         <v>0.9088504577822991</v>
       </c>
       <c r="K7" s="38" t="n">
-        <v>0.05070785070785071</v>
+        <v>0.05460088691796009</v>
       </c>
       <c r="L7" s="38" t="n">
-        <v>0.02406989807877274</v>
+        <v>0.02425466584677534</v>
       </c>
     </row>
     <row r="8">
@@ -47630,31 +47644,31 @@
         </is>
       </c>
       <c r="D9" s="37" t="n">
-        <v>1795</v>
+        <v>1518</v>
       </c>
       <c r="E9" s="37" t="n">
-        <v>7750</v>
+        <v>7159</v>
       </c>
       <c r="F9" s="37" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G9" s="38" t="n">
-        <v>116932</v>
+        <v>115047</v>
       </c>
       <c r="H9" s="38" t="n">
-        <v>6576.18745390356</v>
+        <v>6486.140157229423</v>
       </c>
       <c r="I9" s="38" t="n">
-        <v>0.6866870696250956</v>
+        <v>0.6495507060333762</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>0.9171000617553824</v>
+        <v>0.9158560700306643</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>0.462033462033462</v>
+        <v>0.4207317073170732</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>0.4725556282986995</v>
+        <v>0.4685068068626533</v>
       </c>
     </row>
     <row r="10">
@@ -47684,10 +47698,10 @@
         <v>602.9797559024207</v>
       </c>
       <c r="I10" s="38" t="n">
-        <v>0.3133129303749044</v>
+        <v>0.3504492939666239</v>
       </c>
       <c r="J10" s="38" t="n">
-        <v>0.08289993824461755</v>
+        <v>0.08414392996933574</v>
       </c>
       <c r="K10" s="38" t="n">
         <v>0.5652173913043478</v>
@@ -47729,10 +47743,10 @@
         <v>0.9590140233456422</v>
       </c>
       <c r="K11" s="38" t="n">
-        <v>0.1724581724581725</v>
+        <v>0.1856984478935698</v>
       </c>
       <c r="L11" s="38" t="n">
-        <v>0.1558158143594966</v>
+        <v>0.1570119033559889</v>
       </c>
     </row>
     <row r="12">
@@ -47807,10 +47821,10 @@
         <v>0.7674680510049218</v>
       </c>
       <c r="K13" s="38" t="n">
-        <v>0.06229086229086229</v>
+        <v>0.06707317073170732</v>
       </c>
       <c r="L13" s="38" t="n">
-        <v>0.06833410117763067</v>
+        <v>0.06885865426513167</v>
       </c>
     </row>
     <row r="14">
@@ -47976,7 +47990,7 @@
         <v>1564</v>
       </c>
       <c r="D3" s="37" t="n">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="E3" s="38" t="n">
         <v>80.1864183716965</v>
@@ -48000,7 +48014,7 @@
         <v>277.6970748125938</v>
       </c>
       <c r="L3" s="38" t="n">
-        <v>2.190476190476191</v>
+        <v>2.238636363636364</v>
       </c>
       <c r="M3" s="37" t="n">
         <v>34</v>
@@ -48019,34 +48033,34 @@
         </is>
       </c>
       <c r="C4" s="37" t="n">
-        <v>3762</v>
+        <v>3782</v>
       </c>
       <c r="D4" s="37" t="n">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="E4" s="38" t="n">
-        <v>37.66246002210915</v>
+        <v>41.32553532606415</v>
       </c>
       <c r="F4" s="38" t="n">
         <v>11</v>
       </c>
       <c r="G4" s="38" t="n">
-        <v>1.91843572397052</v>
+        <v>2.130173049332918</v>
       </c>
       <c r="H4" s="38" t="n">
-        <v>0.530985</v>
+        <v>0.5379085</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>4.350877192982456</v>
+        <v>4.333950290851401</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>4.443115364167996</v>
+        <v>4.426493918561608</v>
       </c>
       <c r="K4" s="38" t="n">
-        <v>270.3707068077138</v>
+        <v>287.7181054454293</v>
       </c>
       <c r="L4" s="38" t="n">
-        <v>2.402298850574712</v>
+        <v>2.450617283950617</v>
       </c>
       <c r="M4" s="37" t="n">
         <v>60</v>
@@ -48055,7 +48069,7 @@
         <v>6</v>
       </c>
       <c r="O4" s="38" t="n">
-        <v>0.2693118659066443</v>
+        <v>0.272943114847685</v>
       </c>
     </row>
   </sheetData>
@@ -48178,10 +48192,10 @@
         </is>
       </c>
       <c r="D6" s="38" t="n">
-        <v>68747</v>
+        <v>75857</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.4852061267977776</v>
+        <v>0.4853506891302162</v>
       </c>
     </row>
     <row r="7">
@@ -48196,10 +48210,10 @@
         </is>
       </c>
       <c r="D7" s="38" t="n">
-        <v>12218.1746031746</v>
+        <v>15268.1746031746</v>
       </c>
       <c r="E7" s="38" t="n">
-        <v>0.08623406367907432</v>
+        <v>0.09768932419435593</v>
       </c>
     </row>
     <row r="8">
@@ -48214,10 +48228,10 @@
         </is>
       </c>
       <c r="D8" s="38" t="n">
-        <v>60721</v>
+        <v>65168</v>
       </c>
       <c r="E8" s="38" t="n">
-        <v>0.428559809523148</v>
+        <v>0.4169599866754278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add part2 and part3 to codebase
</commit_message>
<xml_diff>
--- a/outputs/round2/summary_tables.xlsx
+++ b/outputs/round2/summary_tables.xlsx
@@ -17,6 +17,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1.3 Segment Profile" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1.3 Packaging" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1.3 Geo Spread" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2.2 Safety Stock" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2.2 Lead Time Sensitivity" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2.2 Inventory Pooling" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2.1 HCM Districts" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Q1.1 Full SKU Ranking'!$B$2:$Q$472</definedName>
@@ -28,6 +32,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Q1.3 Segment Profile'!$B$2:$O$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Q1.3 Packaging'!$B$2:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Q1.3 Geo Spread'!$B$2:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Q2.2 Safety Stock'!$B$2:$O$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Q2.2 Lead Time Sensitivity'!$B$2:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Q2.2 Inventory Pooling'!$B$2:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Q2.1 HCM Districts'!$B$2:$I$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1903,6 +1911,2494 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:O30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QUESTION 2.2 — CLASS A SAFETY STOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>sku_code</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>mu_monthly</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>sigma_monthly</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>mu_daily</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>sigma_daily</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>ss_b2b</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>rop_b2b</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>ss_b2c</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>rop_b2c</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>product_name</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>abc_quantity</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>xyz_frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>4200009163</t>
+        </is>
+      </c>
+      <c r="C3" s="38" t="n">
+        <v>7738.142857142857</v>
+      </c>
+      <c r="D3" s="38" t="n">
+        <v>7579.496078864597</v>
+      </c>
+      <c r="E3" s="38" t="n">
+        <v>257.9380952380952</v>
+      </c>
+      <c r="F3" s="38" t="n">
+        <v>1383.820325638698</v>
+      </c>
+      <c r="G3" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H3" s="38" t="n">
+        <v>5107.804608168952</v>
+      </c>
+      <c r="I3" s="38" t="n">
+        <v>6397.495084359428</v>
+      </c>
+      <c r="J3" s="38" t="n">
+        <v>3226.276732248457</v>
+      </c>
+      <c r="K3" s="38" t="n">
+        <v>3742.152922724648</v>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>Quạt lửng ASIAVINA - VY628890 - Đen</t>
+        </is>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>4200008102</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="n">
+        <v>1811</v>
+      </c>
+      <c r="D4" s="38" t="n">
+        <v>2780.610484527933</v>
+      </c>
+      <c r="E4" s="38" t="n">
+        <v>60.36666666666667</v>
+      </c>
+      <c r="F4" s="38" t="n">
+        <v>507.6676953371062</v>
+      </c>
+      <c r="G4" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H4" s="38" t="n">
+        <v>1870.008751152734</v>
+      </c>
+      <c r="I4" s="38" t="n">
+        <v>2171.842084486067</v>
+      </c>
+      <c r="J4" s="38" t="n">
+        <v>1182.071877644764</v>
+      </c>
+      <c r="K4" s="38" t="n">
+        <v>1302.805210978098</v>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>Quạt lửng ASIAvina - VY538790 - Xám</t>
+        </is>
+      </c>
+      <c r="M4" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N4" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O4" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>4200009000</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="n">
+        <v>1932.857142857143</v>
+      </c>
+      <c r="D5" s="38" t="n">
+        <v>2352.359059084549</v>
+      </c>
+      <c r="E5" s="38" t="n">
+        <v>64.42857142857143</v>
+      </c>
+      <c r="F5" s="38" t="n">
+        <v>429.4800400040784</v>
+      </c>
+      <c r="G5" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H5" s="38" t="n">
+        <v>1583.321314292101</v>
+      </c>
+      <c r="I5" s="38" t="n">
+        <v>1905.464171434958</v>
+      </c>
+      <c r="J5" s="38" t="n">
+        <v>1000.538670258635</v>
+      </c>
+      <c r="K5" s="38" t="n">
+        <v>1129.395813115778</v>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng ASIAVINA Turbo X - VY629890 - Đen</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O5" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>4100000722</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="n">
+        <v>994.2857142857143</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>1521.760024257626</v>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>33.14285714285715</v>
+      </c>
+      <c r="F6" s="38" t="n">
+        <v>277.8340974651703</v>
+      </c>
+      <c r="G6" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H6" s="38" t="n">
+        <v>1023.419239650838</v>
+      </c>
+      <c r="I6" s="38" t="n">
+        <v>1189.133525365124</v>
+      </c>
+      <c r="J6" s="38" t="n">
+        <v>646.9226472113958</v>
+      </c>
+      <c r="K6" s="38" t="n">
+        <v>713.2083614971101</v>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng Tefal - VF2820F0 - đen</t>
+        </is>
+      </c>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N6" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O6" s="12" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>4200000163</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="n">
+        <v>1531</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <v>1318.179679204116</v>
+      </c>
+      <c r="E7" s="38" t="n">
+        <v>51.03333333333333</v>
+      </c>
+      <c r="F7" s="38" t="n">
+        <v>240.665581715006</v>
+      </c>
+      <c r="G7" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H7" s="38" t="n">
+        <v>889.2195241747893</v>
+      </c>
+      <c r="I7" s="38" t="n">
+        <v>1144.386190841456</v>
+      </c>
+      <c r="J7" s="38" t="n">
+        <v>561.4511632296717</v>
+      </c>
+      <c r="K7" s="38" t="n">
+        <v>663.5178298963383</v>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>Quạt trần đảo ASIAvina - X16001-XV0 - Xám</t>
+        </is>
+      </c>
+      <c r="M7" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>4200008999</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>1334.095238095238</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>1123.64311116557</v>
+      </c>
+      <c r="E8" s="38" t="n">
+        <v>44.46984126984127</v>
+      </c>
+      <c r="F8" s="38" t="n">
+        <v>205.1482261902225</v>
+      </c>
+      <c r="G8" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H8" s="38" t="n">
+        <v>758.1407575706685</v>
+      </c>
+      <c r="I8" s="38" t="n">
+        <v>980.4899639198748</v>
+      </c>
+      <c r="J8" s="38" t="n">
+        <v>478.6525478288111</v>
+      </c>
+      <c r="K8" s="38" t="n">
+        <v>567.5922303684937</v>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng ASIAVINA Turbo X - VY629790 - Xám</t>
+        </is>
+      </c>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O8" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>4100000838</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="n">
+        <v>393.1428571428572</v>
+      </c>
+      <c r="D9" s="38" t="n">
+        <v>1039.276579897675</v>
+      </c>
+      <c r="E9" s="38" t="n">
+        <v>13.10476190476191</v>
+      </c>
+      <c r="F9" s="38" t="n">
+        <v>189.745075432259</v>
+      </c>
+      <c r="G9" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H9" s="38" t="n">
+        <v>698.2781889153412</v>
+      </c>
+      <c r="I9" s="38" t="n">
+        <v>763.8019984391507</v>
+      </c>
+      <c r="J9" s="38" t="n">
+        <v>441.5509753730466</v>
+      </c>
+      <c r="K9" s="38" t="n">
+        <v>467.7604991825705</v>
+      </c>
+      <c r="L9" s="12" t="inlineStr"/>
+      <c r="M9" s="12" t="inlineStr"/>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>1830009179</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="n">
+        <v>361.2857142857143</v>
+      </c>
+      <c r="D10" s="38" t="n">
+        <v>954.1089585377053</v>
+      </c>
+      <c r="E10" s="38" t="n">
+        <v>12.04285714285714</v>
+      </c>
+      <c r="F10" s="38" t="n">
+        <v>174.1956663029542</v>
+      </c>
+      <c r="G10" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H10" s="38" t="n">
+        <v>641.0556371908283</v>
+      </c>
+      <c r="I10" s="38" t="n">
+        <v>701.269922905114</v>
+      </c>
+      <c r="J10" s="38" t="n">
+        <v>405.3665792873384</v>
+      </c>
+      <c r="K10" s="38" t="n">
+        <v>429.4522935730527</v>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>Bàn ủi khô tích hợp bình xịt nước Tefal FS3120L0</t>
+        </is>
+      </c>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>SDA</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>4200009382</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="n">
+        <v>750.4285714285714</v>
+      </c>
+      <c r="D11" s="38" t="n">
+        <v>913.551103686936</v>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>25.01428571428572</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>166.7908489743586</v>
+      </c>
+      <c r="G11" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H11" s="38" t="n">
+        <v>614.8904623110842</v>
+      </c>
+      <c r="I11" s="38" t="n">
+        <v>739.9618908825128</v>
+      </c>
+      <c r="J11" s="38" t="n">
+        <v>388.5641934077535</v>
+      </c>
+      <c r="K11" s="38" t="n">
+        <v>438.5927648363249</v>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>Quạt sàn ASIAVINA TURBO MAX - VY646990 - Xám</t>
+        </is>
+      </c>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>4200007859</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="n">
+        <v>747.8571428571429</v>
+      </c>
+      <c r="D12" s="38" t="n">
+        <v>766.771897540033</v>
+      </c>
+      <c r="E12" s="38" t="n">
+        <v>24.92857142857143</v>
+      </c>
+      <c r="F12" s="38" t="n">
+        <v>139.992754914572</v>
+      </c>
+      <c r="G12" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H12" s="38" t="n">
+        <v>516.5700516205426</v>
+      </c>
+      <c r="I12" s="38" t="n">
+        <v>641.2129087633997</v>
+      </c>
+      <c r="J12" s="38" t="n">
+        <v>326.3213217582672</v>
+      </c>
+      <c r="K12" s="38" t="n">
+        <v>376.17846461541</v>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng ASIAvina - VY639990 - Xám</t>
+        </is>
+      </c>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>4200008101</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="n">
+        <v>978.7142857142857</v>
+      </c>
+      <c r="D13" s="38" t="n">
+        <v>751.6809416868556</v>
+      </c>
+      <c r="E13" s="38" t="n">
+        <v>32.62380952380952</v>
+      </c>
+      <c r="F13" s="38" t="n">
+        <v>137.2375359362054</v>
+      </c>
+      <c r="G13" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H13" s="38" t="n">
+        <v>507.6498232968328</v>
+      </c>
+      <c r="I13" s="38" t="n">
+        <v>670.7688709158804</v>
+      </c>
+      <c r="J13" s="38" t="n">
+        <v>320.3924603055104</v>
+      </c>
+      <c r="K13" s="38" t="n">
+        <v>385.6400793531295</v>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>Quạt lửng ASIAvina - VY538990 - Đen</t>
+        </is>
+      </c>
+      <c r="M13" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N13" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>4200008113</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="n">
+        <v>625.4285714285714</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>673.4606786697244</v>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>20.84761904761905</v>
+      </c>
+      <c r="F14" s="38" t="n">
+        <v>122.9565351000488</v>
+      </c>
+      <c r="G14" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>453.5732784728518</v>
+      </c>
+      <c r="I14" s="38" t="n">
+        <v>557.811373710947</v>
+      </c>
+      <c r="J14" s="38" t="n">
+        <v>286.5572759205876</v>
+      </c>
+      <c r="K14" s="38" t="n">
+        <v>328.2525140158257</v>
+      </c>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng ASIAvina - VY539790 - Xám</t>
+        </is>
+      </c>
+      <c r="M14" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O14" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>4200008737</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="n">
+        <v>640.5714285714286</v>
+      </c>
+      <c r="D15" s="38" t="n">
+        <v>669.5677354689012</v>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>21.35238095238095</v>
+      </c>
+      <c r="F15" s="38" t="n">
+        <v>122.2457841646564</v>
+      </c>
+      <c r="G15" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H15" s="38" t="n">
+        <v>451.0303312818577</v>
+      </c>
+      <c r="I15" s="38" t="n">
+        <v>557.7922360437625</v>
+      </c>
+      <c r="J15" s="38" t="n">
+        <v>284.9320665759161</v>
+      </c>
+      <c r="K15" s="38" t="n">
+        <v>327.6368284806779</v>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAVINA VY357792 - 55W Xám</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N15" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>4200007858</t>
+        </is>
+      </c>
+      <c r="C16" s="38" t="n">
+        <v>1067</v>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>646.7977530367073</v>
+      </c>
+      <c r="E16" s="38" t="n">
+        <v>35.56666666666667</v>
+      </c>
+      <c r="F16" s="38" t="n">
+        <v>118.08857316062</v>
+      </c>
+      <c r="G16" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H16" s="38" t="n">
+        <v>438.2915456617699</v>
+      </c>
+      <c r="I16" s="38" t="n">
+        <v>616.1248789951032</v>
+      </c>
+      <c r="J16" s="38" t="n">
+        <v>276.272199681273</v>
+      </c>
+      <c r="K16" s="38" t="n">
+        <v>347.4055330146063</v>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>Quạt sàn ASIAvina - VY636790 - Xám</t>
+        </is>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O16" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>4200009226</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="n">
+        <v>384.1428571428572</v>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>626.8546957021297</v>
+      </c>
+      <c r="E17" s="38" t="n">
+        <v>12.80476190476191</v>
+      </c>
+      <c r="F17" s="38" t="n">
+        <v>114.4474857046977</v>
+      </c>
+      <c r="G17" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H17" s="38" t="n">
+        <v>421.5024714616814</v>
+      </c>
+      <c r="I17" s="38" t="n">
+        <v>485.5262809854909</v>
+      </c>
+      <c r="J17" s="38" t="n">
+        <v>266.4567143423451</v>
+      </c>
+      <c r="K17" s="38" t="n">
+        <v>292.0662381518689</v>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>Quạt lửng ASIAvina - VY358291 - Chuối non</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>4200009001</t>
+        </is>
+      </c>
+      <c r="C18" s="38" t="n">
+        <v>762.8571428571429</v>
+      </c>
+      <c r="D18" s="38" t="n">
+        <v>616.7547942176666</v>
+      </c>
+      <c r="E18" s="38" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="F18" s="38" t="n">
+        <v>112.6035044141576</v>
+      </c>
+      <c r="G18" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H18" s="38" t="n">
+        <v>416.2999334681134</v>
+      </c>
+      <c r="I18" s="38" t="n">
+        <v>543.4427906109705</v>
+      </c>
+      <c r="J18" s="38" t="n">
+        <v>262.7922972752859</v>
+      </c>
+      <c r="K18" s="38" t="n">
+        <v>313.6494401324287</v>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAVINA Turbo X - VY627790 - Xám</t>
+        </is>
+      </c>
+      <c r="M18" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O18" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>4200000164</t>
+        </is>
+      </c>
+      <c r="C19" s="38" t="n">
+        <v>668.4285714285714</v>
+      </c>
+      <c r="D19" s="38" t="n">
+        <v>524.3131561522042</v>
+      </c>
+      <c r="E19" s="38" t="n">
+        <v>22.28095238095238</v>
+      </c>
+      <c r="F19" s="38" t="n">
+        <v>95.72604760709693</v>
+      </c>
+      <c r="G19" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H19" s="38" t="n">
+        <v>354.0146319193992</v>
+      </c>
+      <c r="I19" s="38" t="n">
+        <v>465.4193938241611</v>
+      </c>
+      <c r="J19" s="38" t="n">
+        <v>223.4480625268586</v>
+      </c>
+      <c r="K19" s="38" t="n">
+        <v>268.0099672887634</v>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>Quạt trần đảo ASIAvina - X16002-XV0 - Xám</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N19" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>4100000738</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="n">
+        <v>445.7142857142857</v>
+      </c>
+      <c r="D20" s="38" t="n">
+        <v>467.8624136380674</v>
+      </c>
+      <c r="E20" s="38" t="n">
+        <v>14.85714285714286</v>
+      </c>
+      <c r="F20" s="38" t="n">
+        <v>85.41959925279406</v>
+      </c>
+      <c r="G20" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H20" s="38" t="n">
+        <v>315.150722741428</v>
+      </c>
+      <c r="I20" s="38" t="n">
+        <v>389.4364370271423</v>
+      </c>
+      <c r="J20" s="38" t="n">
+        <v>199.093933051155</v>
+      </c>
+      <c r="K20" s="38" t="n">
+        <v>228.8082187654407</v>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>Quạt đứng - TEFAL - VF4420F2 - đen</t>
+        </is>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O20" s="12" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>4200008122</t>
+        </is>
+      </c>
+      <c r="C21" s="38" t="n">
+        <v>562.2857142857143</v>
+      </c>
+      <c r="D21" s="38" t="n">
+        <v>424.5439570039496</v>
+      </c>
+      <c r="E21" s="38" t="n">
+        <v>18.74285714285714</v>
+      </c>
+      <c r="F21" s="38" t="n">
+        <v>77.51076730118885</v>
+      </c>
+      <c r="G21" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H21" s="38" t="n">
+        <v>286.7725717849715</v>
+      </c>
+      <c r="I21" s="38" t="n">
+        <v>380.4868574992573</v>
+      </c>
+      <c r="J21" s="38" t="n">
+        <v>180.9773779721285</v>
+      </c>
+      <c r="K21" s="38" t="n">
+        <v>218.4630922578428</v>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAvina - VY377790 - Xám</t>
+        </is>
+      </c>
+      <c r="M21" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N21" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O21" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>4200008736</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="n">
+        <v>363.1428571428572</v>
+      </c>
+      <c r="D22" s="38" t="n">
+        <v>420.4439830193112</v>
+      </c>
+      <c r="E22" s="38" t="n">
+        <v>12.10476190476191</v>
+      </c>
+      <c r="F22" s="38" t="n">
+        <v>76.76221788899859</v>
+      </c>
+      <c r="G22" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H22" s="38" t="n">
+        <v>283.0581654044113</v>
+      </c>
+      <c r="I22" s="38" t="n">
+        <v>343.5819749282209</v>
+      </c>
+      <c r="J22" s="38" t="n">
+        <v>178.8555138876847</v>
+      </c>
+      <c r="K22" s="38" t="n">
+        <v>203.0650376972085</v>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAVINA VY357192 - 55W Xanh Thiên Thanh</t>
+        </is>
+      </c>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>4200009023</t>
+        </is>
+      </c>
+      <c r="C23" s="38" t="n">
+        <v>419.8571428571428</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <v>407.0075464375849</v>
+      </c>
+      <c r="E23" s="38" t="n">
+        <v>13.9952380952381</v>
+      </c>
+      <c r="F23" s="38" t="n">
+        <v>74.30907141956556</v>
+      </c>
+      <c r="G23" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H23" s="38" t="n">
+        <v>274.3012574093693</v>
+      </c>
+      <c r="I23" s="38" t="n">
+        <v>344.2774478855598</v>
+      </c>
+      <c r="J23" s="38" t="n">
+        <v>173.2540588351115</v>
+      </c>
+      <c r="K23" s="38" t="n">
+        <v>201.2445350255877</v>
+      </c>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAVINA - VY377092 - 55W Xám</t>
+        </is>
+      </c>
+      <c r="M23" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N23" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O23" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>4200008229</t>
+        </is>
+      </c>
+      <c r="C24" s="38" t="n">
+        <v>801.1428571428571</v>
+      </c>
+      <c r="D24" s="38" t="n">
+        <v>387.7049688321558</v>
+      </c>
+      <c r="E24" s="38" t="n">
+        <v>26.7047619047619</v>
+      </c>
+      <c r="F24" s="38" t="n">
+        <v>70.78491902873635</v>
+      </c>
+      <c r="G24" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H24" s="38" t="n">
+        <v>264.0502642846202</v>
+      </c>
+      <c r="I24" s="38" t="n">
+        <v>397.5740738084297</v>
+      </c>
+      <c r="J24" s="38" t="n">
+        <v>166.1311195364807</v>
+      </c>
+      <c r="K24" s="38" t="n">
+        <v>219.5406433460045</v>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAvina - VY377990 - Xám</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>4200009002</t>
+        </is>
+      </c>
+      <c r="C25" s="38" t="n">
+        <v>427.7142857142857</v>
+      </c>
+      <c r="D25" s="38" t="n">
+        <v>389.2581466866233</v>
+      </c>
+      <c r="E25" s="38" t="n">
+        <v>14.25714285714286</v>
+      </c>
+      <c r="F25" s="38" t="n">
+        <v>71.06848921097281</v>
+      </c>
+      <c r="G25" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H25" s="38" t="n">
+        <v>262.4634328775895</v>
+      </c>
+      <c r="I25" s="38" t="n">
+        <v>333.7491471633037</v>
+      </c>
+      <c r="J25" s="38" t="n">
+        <v>165.7477449554158</v>
+      </c>
+      <c r="K25" s="38" t="n">
+        <v>194.2620306697015</v>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>QUẠT treo ASIAVINA TURBO VY627890</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>4200008372</t>
+        </is>
+      </c>
+      <c r="C26" s="38" t="n">
+        <v>529.2857142857143</v>
+      </c>
+      <c r="D26" s="38" t="n">
+        <v>381.7528494919692</v>
+      </c>
+      <c r="E26" s="38" t="n">
+        <v>17.64285714285715</v>
+      </c>
+      <c r="F26" s="38" t="n">
+        <v>69.6982156862087</v>
+      </c>
+      <c r="G26" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H26" s="38" t="n">
+        <v>258.0106686115152</v>
+      </c>
+      <c r="I26" s="38" t="n">
+        <v>346.2249543258009</v>
+      </c>
+      <c r="J26" s="38" t="n">
+        <v>162.7926786468204</v>
+      </c>
+      <c r="K26" s="38" t="n">
+        <v>198.0783929325347</v>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>QUẠT SÀN TURBO VY616990</t>
+        </is>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>4200008366</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="n">
+        <v>405.4285714285714</v>
+      </c>
+      <c r="D27" s="38" t="n">
+        <v>349.7055223769742</v>
+      </c>
+      <c r="E27" s="38" t="n">
+        <v>13.51428571428571</v>
+      </c>
+      <c r="F27" s="38" t="n">
+        <v>63.84720102999879</v>
+      </c>
+      <c r="G27" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H27" s="38" t="n">
+        <v>235.9010373926839</v>
+      </c>
+      <c r="I27" s="38" t="n">
+        <v>303.4724659641125</v>
+      </c>
+      <c r="J27" s="38" t="n">
+        <v>148.9482701243213</v>
+      </c>
+      <c r="K27" s="38" t="n">
+        <v>175.9768415528927</v>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>QUẠT SÀN TURB0 VY616790</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>4200008371</t>
+        </is>
+      </c>
+      <c r="C28" s="38" t="n">
+        <v>479.2857142857143</v>
+      </c>
+      <c r="D28" s="38" t="n">
+        <v>340.8101691977096</v>
+      </c>
+      <c r="E28" s="38" t="n">
+        <v>15.97619047619048</v>
+      </c>
+      <c r="F28" s="38" t="n">
+        <v>62.22313916557929</v>
+      </c>
+      <c r="G28" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H28" s="38" t="n">
+        <v>230.3812598278365</v>
+      </c>
+      <c r="I28" s="38" t="n">
+        <v>310.2622122087889</v>
+      </c>
+      <c r="J28" s="38" t="n">
+        <v>145.349948819531</v>
+      </c>
+      <c r="K28" s="38" t="n">
+        <v>177.302329771912</v>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>QUẠT ĐỨNG VY619990</t>
+        </is>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>4200008117</t>
+        </is>
+      </c>
+      <c r="C29" s="38" t="n">
+        <v>576.1428571428571</v>
+      </c>
+      <c r="D29" s="38" t="n">
+        <v>318.8366502204687</v>
+      </c>
+      <c r="E29" s="38" t="n">
+        <v>19.2047619047619</v>
+      </c>
+      <c r="F29" s="38" t="n">
+        <v>58.2113418283784</v>
+      </c>
+      <c r="G29" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H29" s="38" t="n">
+        <v>216.4386485788499</v>
+      </c>
+      <c r="I29" s="38" t="n">
+        <v>312.4624581026595</v>
+      </c>
+      <c r="J29" s="38" t="n">
+        <v>136.3399018976154</v>
+      </c>
+      <c r="K29" s="38" t="n">
+        <v>174.7494257071392</v>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAvina - VY357690 - trắng</t>
+        </is>
+      </c>
+      <c r="M29" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>4200009625</t>
+        </is>
+      </c>
+      <c r="C30" s="38" t="n">
+        <v>369.4285714285714</v>
+      </c>
+      <c r="D30" s="38" t="n">
+        <v>306.6414068271804</v>
+      </c>
+      <c r="E30" s="38" t="n">
+        <v>12.31428571428571</v>
+      </c>
+      <c r="F30" s="38" t="n">
+        <v>55.98480519478846</v>
+      </c>
+      <c r="G30" s="38" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="H30" s="38" t="n">
+        <v>206.9246127460702</v>
+      </c>
+      <c r="I30" s="38" t="n">
+        <v>268.4960413174987</v>
+      </c>
+      <c r="J30" s="38" t="n">
+        <v>130.635241174403</v>
+      </c>
+      <c r="K30" s="38" t="n">
+        <v>155.2638126029744</v>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>Quạt treo ASIAVINA - VY617090 - Đen</t>
+        </is>
+      </c>
+      <c r="M30" s="12" t="inlineStr">
+        <is>
+          <t>Fan</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:O30"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QUESTION 2.2 — LEAD TIME SENSITIVITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>lead_time_days</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>total_safety_stock</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>delta_from_lt2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="38" t="n">
+        <v>12340.20950413805</v>
+      </c>
+      <c r="D3" s="38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="38" t="n">
+        <v>15113.60830209082</v>
+      </c>
+      <c r="D4" s="38" t="n">
+        <v>2773.398797952768</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="38" t="n">
+        <v>17451.6916432774</v>
+      </c>
+      <c r="D5" s="38" t="n">
+        <v>5111.482139139345</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="38" t="n">
+        <v>19511.58441836664</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>7171.374914228585</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="38" t="n">
+        <v>21373.86983721144</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <v>9033.660333073392</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>23086.41802274807</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>10746.20851861002</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:D8"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QUESTION 2.2 — INVENTORY POOLING SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>formula</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>total_ss</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>savings_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Separated B2B + B2C</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Z * sigma * (sqrt(5) + sqrt(2))</t>
+        </is>
+      </c>
+      <c r="D3" s="38" t="n">
+        <v>31851.79392250469</v>
+      </c>
+      <c r="E3" s="38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Pooled (Shared)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Z * sigma * sqrt(3.5)</t>
+        </is>
+      </c>
+      <c r="D4" s="38" t="n">
+        <v>16324.56273719248</v>
+      </c>
+      <c r="E4" s="38" t="n">
+        <v>0.4874837261314043</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:E4"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QUESTION 2.1 — HCM DISTRICT SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>orders</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>cbm</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>avg_dist_my_phuoc</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>avg_dist_vinh_loc</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>avg_lat</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>avg_lon</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Thủ Đức</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="n">
+        <v>285</v>
+      </c>
+      <c r="D3" s="38" t="n">
+        <v>3532.75</v>
+      </c>
+      <c r="E3" s="38" t="n">
+        <v>191.3269125531167</v>
+      </c>
+      <c r="F3" s="38" t="n">
+        <v>40.13305293476246</v>
+      </c>
+      <c r="G3" s="38" t="n">
+        <v>22.67671958847953</v>
+      </c>
+      <c r="H3" s="38" t="n">
+        <v>10.82520241172214</v>
+      </c>
+      <c r="I3" s="38" t="n">
+        <v>106.765811142547</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Bình Tân</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>249</v>
+      </c>
+      <c r="D4" s="38" t="n">
+        <v>26954.40833333333</v>
+      </c>
+      <c r="E4" s="38" t="n">
+        <v>1690.636797969883</v>
+      </c>
+      <c r="F4" s="38" t="n">
+        <v>41.29724903417543</v>
+      </c>
+      <c r="G4" s="38" t="n">
+        <v>5.339041572400149</v>
+      </c>
+      <c r="H4" s="38" t="n">
+        <v>10.78082397609562</v>
+      </c>
+      <c r="I4" s="38" t="n">
+        <v>106.603704184263</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Tân Phú</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>223</v>
+      </c>
+      <c r="D5" s="38" t="n">
+        <v>23468.58333333333</v>
+      </c>
+      <c r="E5" s="38" t="n">
+        <v>1194.685725449033</v>
+      </c>
+      <c r="F5" s="38" t="n">
+        <v>40.8562235155962</v>
+      </c>
+      <c r="G5" s="38" t="n">
+        <v>7.091543598248473</v>
+      </c>
+      <c r="H5" s="38" t="n">
+        <v>10.78477419805589</v>
+      </c>
+      <c r="I5" s="38" t="n">
+        <v>106.6266994459295</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Quận 10</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>197</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>271.425</v>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>13.99009246692222</v>
+      </c>
+      <c r="F6" s="38" t="n">
+        <v>42.44266797562761</v>
+      </c>
+      <c r="G6" s="38" t="n">
+        <v>11.90646464618847</v>
+      </c>
+      <c r="H6" s="38" t="n">
+        <v>10.77469621621622</v>
+      </c>
+      <c r="I6" s="38" t="n">
+        <v>106.6734668513513</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Quận 12</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>152</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <v>2128.366666666667</v>
+      </c>
+      <c r="E7" s="38" t="n">
+        <v>97.45092171186667</v>
+      </c>
+      <c r="F7" s="38" t="n">
+        <v>32.69929009468674</v>
+      </c>
+      <c r="G7" s="38" t="n">
+        <v>11.48076595025293</v>
+      </c>
+      <c r="H7" s="38" t="n">
+        <v>10.85974060036832</v>
+      </c>
+      <c r="I7" s="38" t="n">
+        <v>106.6363278563536</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Gò Vấp</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>77</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>884.4166666666666</v>
+      </c>
+      <c r="E8" s="38" t="n">
+        <v>39.78345297910001</v>
+      </c>
+      <c r="F8" s="38" t="n">
+        <v>36.17068743010955</v>
+      </c>
+      <c r="G8" s="38" t="n">
+        <v>12.40636170472616</v>
+      </c>
+      <c r="H8" s="38" t="n">
+        <v>10.83137770663265</v>
+      </c>
+      <c r="I8" s="38" t="n">
+        <v>106.6672134591837</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Quận 1</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>58</v>
+      </c>
+      <c r="D9" s="38" t="n">
+        <v>675.6458333333334</v>
+      </c>
+      <c r="E9" s="38" t="n">
+        <v>38.9121978145</v>
+      </c>
+      <c r="F9" s="38" t="n">
+        <v>43.05721898216862</v>
+      </c>
+      <c r="G9" s="38" t="n">
+        <v>14.63005386805622</v>
+      </c>
+      <c r="H9" s="38" t="n">
+        <v>10.77354887903226</v>
+      </c>
+      <c r="I9" s="38" t="n">
+        <v>106.6981529112903</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Quận 7</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="n">
+        <v>51</v>
+      </c>
+      <c r="D10" s="38" t="n">
+        <v>1439.25</v>
+      </c>
+      <c r="E10" s="38" t="n">
+        <v>55.64606078265</v>
+      </c>
+      <c r="F10" s="38" t="n">
+        <v>47.8531259868564</v>
+      </c>
+      <c r="G10" s="38" t="n">
+        <v>18.24661145345621</v>
+      </c>
+      <c r="H10" s="38" t="n">
+        <v>10.73518596341463</v>
+      </c>
+      <c r="I10" s="38" t="n">
+        <v>106.7240696443089</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Bình Chánh</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="n">
+        <v>49</v>
+      </c>
+      <c r="D11" s="38" t="n">
+        <v>543.5</v>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>23.75929453625</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>45.21387782210643</v>
+      </c>
+      <c r="G11" s="38" t="n">
+        <v>10.13160210576056</v>
+      </c>
+      <c r="H11" s="38" t="n">
+        <v>10.75013204255319</v>
+      </c>
+      <c r="I11" s="38" t="n">
+        <v>106.6199481702128</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Quận 3</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="38" t="n">
+        <v>1101.118055555556</v>
+      </c>
+      <c r="E12" s="38" t="n">
+        <v>38.54646990452778</v>
+      </c>
+      <c r="F12" s="38" t="n">
+        <v>41.19451007037444</v>
+      </c>
+      <c r="G12" s="38" t="n">
+        <v>11.71154122648066</v>
+      </c>
+      <c r="H12" s="38" t="n">
+        <v>10.78585066363636</v>
+      </c>
+      <c r="I12" s="38" t="n">
+        <v>106.6722063151515</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Hóc Môn</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="n">
+        <v>27</v>
+      </c>
+      <c r="D13" s="38" t="n">
+        <v>393</v>
+      </c>
+      <c r="E13" s="38" t="n">
+        <v>22.36434343093334</v>
+      </c>
+      <c r="F13" s="38" t="n">
+        <v>29.92431178395903</v>
+      </c>
+      <c r="G13" s="38" t="n">
+        <v>11.85738550677496</v>
+      </c>
+      <c r="H13" s="38" t="n">
+        <v>10.88301146808511</v>
+      </c>
+      <c r="I13" s="38" t="n">
+        <v>106.6076619787234</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Quận 4</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>23</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>1086</v>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>33.87651122953334</v>
+      </c>
+      <c r="F14" s="38" t="n">
+        <v>44.45704370253569</v>
+      </c>
+      <c r="G14" s="38" t="n">
+        <v>15.0212149451197</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>10.761065</v>
+      </c>
+      <c r="I14" s="38" t="n">
+        <v>106.700337</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Củ Chi</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="n">
+        <v>21</v>
+      </c>
+      <c r="D15" s="38" t="n">
+        <v>182</v>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>8.546705433333333</v>
+      </c>
+      <c r="F15" s="38" t="n">
+        <v>23.80879759782039</v>
+      </c>
+      <c r="G15" s="38" t="n">
+        <v>22.11641099445494</v>
+      </c>
+      <c r="H15" s="38" t="n">
+        <v>10.972192</v>
+      </c>
+      <c r="I15" s="38" t="n">
+        <v>106.496543</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Quận 5</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>2304</v>
+      </c>
+      <c r="E16" s="38" t="n">
+        <v>79.290767876</v>
+      </c>
+      <c r="F16" s="38" t="n">
+        <v>44.63275893481413</v>
+      </c>
+      <c r="G16" s="38" t="n">
+        <v>11.38323740582554</v>
+      </c>
+      <c r="H16" s="38" t="n">
+        <v>10.75352</v>
+      </c>
+      <c r="I16" s="38" t="n">
+        <v>106.664158</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Phú Nhuận</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>78.16666666666667</v>
+      </c>
+      <c r="E17" s="38" t="n">
+        <v>4.868871250000001</v>
+      </c>
+      <c r="F17" s="38" t="n">
+        <v>39.37651319044713</v>
+      </c>
+      <c r="G17" s="38" t="n">
+        <v>12.85524277948338</v>
+      </c>
+      <c r="H17" s="38" t="n">
+        <v>10.803877</v>
+      </c>
+      <c r="I17" s="38" t="n">
+        <v>106.681113</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Quận 6</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="38" t="n">
+        <v>83.66666666666667</v>
+      </c>
+      <c r="E18" s="38" t="n">
+        <v>3.672757857916667</v>
+      </c>
+      <c r="F18" s="38" t="n">
+        <v>45.52954764545309</v>
+      </c>
+      <c r="G18" s="38" t="n">
+        <v>9.183568180194309</v>
+      </c>
+      <c r="H18" s="38" t="n">
+        <v>10.74325171428571</v>
+      </c>
+      <c r="I18" s="38" t="n">
+        <v>106.6367877142857</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Nhà Bè</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="38" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E19" s="38" t="n">
+        <v>0.8754587575</v>
+      </c>
+      <c r="F19" s="38" t="n">
+        <v>54.81212903337548</v>
+      </c>
+      <c r="G19" s="38" t="n">
+        <v>23.78703100843765</v>
+      </c>
+      <c r="H19" s="38" t="n">
+        <v>10.678244</v>
+      </c>
+      <c r="I19" s="38" t="n">
+        <v>106.75368</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Bình Thạnh</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="38" t="n">
+        <v>216</v>
+      </c>
+      <c r="E20" s="38" t="n">
+        <v>10.422910692</v>
+      </c>
+      <c r="F20" s="38" t="n">
+        <v>41.05386007300064</v>
+      </c>
+      <c r="G20" s="38" t="n">
+        <v>16.7152510238936</v>
+      </c>
+      <c r="H20" s="38" t="n">
+        <v>10.79665713333333</v>
+      </c>
+      <c r="I20" s="38" t="n">
+        <v>106.7170754</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Quận 11</t>
+        </is>
+      </c>
+      <c r="C21" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="38" t="n">
+        <v>36.47916666666666</v>
+      </c>
+      <c r="E21" s="38" t="n">
+        <v>1.831972858333333</v>
+      </c>
+      <c r="F21" s="38" t="n">
+        <v>44.26656933521375</v>
+      </c>
+      <c r="G21" s="38" t="n">
+        <v>9.681097357182818</v>
+      </c>
+      <c r="H21" s="38" t="n">
+        <v>10.755245</v>
+      </c>
+      <c r="I21" s="38" t="n">
+        <v>106.648289</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Quận 8</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="38" t="n">
+        <v>24</v>
+      </c>
+      <c r="E22" s="38" t="n">
+        <v>1.581365</v>
+      </c>
+      <c r="F22" s="38" t="n">
+        <v>46.0207362739435</v>
+      </c>
+      <c r="G22" s="38" t="n">
+        <v>13.18427804057327</v>
+      </c>
+      <c r="H22" s="38" t="n">
+        <v>10.742739</v>
+      </c>
+      <c r="I22" s="38" t="n">
+        <v>106.677766</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Tân Bình</t>
+        </is>
+      </c>
+      <c r="C23" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" s="38" t="n">
+        <v>7.101685000000001</v>
+      </c>
+      <c r="F23" s="38" t="n">
+        <v>41.20473766650456</v>
+      </c>
+      <c r="G23" s="38" t="n">
+        <v>8.779682938327934</v>
+      </c>
+      <c r="H23" s="38" t="n">
+        <v>10.782636</v>
+      </c>
+      <c r="I23" s="38" t="n">
+        <v>106.645341</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B2:I23"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix the logic of safety stock calculation in part 2
</commit_message>
<xml_diff>
--- a/outputs/round2/summary_tables.xlsx
+++ b/outputs/round2/summary_tables.xlsx
@@ -33,8 +33,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Q1.3 Packaging'!$B$2:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Q1.3 Geo Spread'!$B$2:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Q2.2 Safety Stock'!$B$2:$O$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Q2.2 Lead Time Sensitivity'!$B$2:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Q2.2 Inventory Pooling'!$B$2:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Q2.2 Lead Time Sensitivity'!$B$2:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Q2.2 Inventory Pooling'!$B$2:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Q2.1 HCM Districts'!$B$2:$I$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1977,22 +1977,22 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>ss_b2b</t>
+          <t>lt_avg</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>rop_b2b</t>
+          <t>sqrt_lt</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>ss_b2c</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>rop_b2c</t>
+          <t>rop</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -2038,16 +2038,16 @@
         <v>1.645</v>
       </c>
       <c r="H3" s="38" t="n">
-        <v>5107.804608168952</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I3" s="38" t="n">
-        <v>6397.495084359428</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J3" s="38" t="n">
-        <v>3226.276732248457</v>
+        <v>3174.470465180855</v>
       </c>
       <c r="K3" s="38" t="n">
-        <v>3742.152922724648</v>
+        <v>3676.081237941402</v>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
@@ -2092,16 +2092,16 @@
         <v>1.645</v>
       </c>
       <c r="H4" s="38" t="n">
-        <v>1870.008751152734</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I4" s="38" t="n">
-        <v>2171.842084486067</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J4" s="38" t="n">
-        <v>1182.071877644764</v>
+        <v>1164.58479118686</v>
       </c>
       <c r="K4" s="38" t="n">
-        <v>1302.805210978098</v>
+        <v>1281.979510596934</v>
       </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
@@ -2146,16 +2146,16 @@
         <v>1.645</v>
       </c>
       <c r="H5" s="38" t="n">
-        <v>1583.321314292101</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I5" s="38" t="n">
-        <v>1905.464171434958</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J5" s="38" t="n">
-        <v>1000.538670258635</v>
+        <v>985.2230648139804</v>
       </c>
       <c r="K5" s="38" t="n">
-        <v>1129.395813115778</v>
+        <v>1110.516947721474</v>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
@@ -2200,16 +2200,16 @@
         <v>1.645</v>
       </c>
       <c r="H6" s="38" t="n">
-        <v>1023.419239650838</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I6" s="38" t="n">
-        <v>1189.133525365124</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>646.9226472113958</v>
+        <v>637.3487368862633</v>
       </c>
       <c r="K6" s="38" t="n">
-        <v>713.2083614971101</v>
+        <v>701.8014660094086</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
@@ -2254,16 +2254,16 @@
         <v>1.645</v>
       </c>
       <c r="H7" s="38" t="n">
-        <v>889.2195241747893</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I7" s="38" t="n">
-        <v>1144.386190841456</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J7" s="38" t="n">
-        <v>561.4511632296717</v>
+        <v>552.0845206455834</v>
       </c>
       <c r="K7" s="38" t="n">
-        <v>663.5178298963383</v>
+        <v>651.3287588658059</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
@@ -2308,16 +2308,16 @@
         <v>1.645</v>
       </c>
       <c r="H8" s="38" t="n">
-        <v>758.1407575706685</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I8" s="38" t="n">
-        <v>980.4899639198748</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J8" s="38" t="n">
-        <v>478.6525478288111</v>
+        <v>470.6080500187236</v>
       </c>
       <c r="K8" s="38" t="n">
-        <v>567.5922303684937</v>
+        <v>557.0883018920014</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
@@ -2362,16 +2362,16 @@
         <v>1.645</v>
       </c>
       <c r="H9" s="38" t="n">
-        <v>698.2781889153412</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I9" s="38" t="n">
-        <v>763.8019984391507</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>441.5509753730466</v>
+        <v>435.2733709090529</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>467.7604991825705</v>
+        <v>460.7581281715379</v>
       </c>
       <c r="L9" s="12" t="inlineStr"/>
       <c r="M9" s="12" t="inlineStr"/>
@@ -2408,16 +2408,16 @@
         <v>1.645</v>
       </c>
       <c r="H10" s="38" t="n">
-        <v>641.0556371908283</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I10" s="38" t="n">
-        <v>701.269922905114</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J10" s="38" t="n">
-        <v>405.3665792873384</v>
+        <v>399.6031765077607</v>
       </c>
       <c r="K10" s="38" t="n">
-        <v>429.4522935730527</v>
+        <v>423.0228535124209</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
@@ -2462,16 +2462,16 @@
         <v>1.645</v>
       </c>
       <c r="H11" s="38" t="n">
-        <v>614.8904623110842</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I11" s="38" t="n">
-        <v>739.9618908825128</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J11" s="38" t="n">
-        <v>388.5641934077535</v>
+        <v>382.6165970550874</v>
       </c>
       <c r="K11" s="38" t="n">
-        <v>438.5927648363249</v>
+        <v>431.2617387338062</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
@@ -2516,16 +2516,16 @@
         <v>1.645</v>
       </c>
       <c r="H12" s="38" t="n">
-        <v>516.5700516205426</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I12" s="38" t="n">
-        <v>641.2129087633997</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J12" s="38" t="n">
-        <v>326.3213217582672</v>
+        <v>321.1420280378509</v>
       </c>
       <c r="K12" s="38" t="n">
-        <v>376.17846461541</v>
+        <v>369.6204816240098</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
@@ -2570,16 +2570,16 @@
         <v>1.645</v>
       </c>
       <c r="H13" s="38" t="n">
-        <v>507.6498232968328</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I13" s="38" t="n">
-        <v>670.7688709158804</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J13" s="38" t="n">
-        <v>320.3924603055104</v>
+        <v>314.8215823052058</v>
       </c>
       <c r="K13" s="38" t="n">
-        <v>385.6400793531295</v>
+        <v>378.2649224234053</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
@@ -2624,16 +2624,16 @@
         <v>1.645</v>
       </c>
       <c r="H14" s="38" t="n">
-        <v>453.5732784728518</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I14" s="38" t="n">
-        <v>557.811373710947</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J14" s="38" t="n">
-        <v>286.5572759205876</v>
+        <v>282.0611042809521</v>
       </c>
       <c r="K14" s="38" t="n">
-        <v>328.2525140158257</v>
+        <v>322.6033525713443</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
         <v>1.645</v>
       </c>
       <c r="H15" s="38" t="n">
-        <v>451.0303312818577</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I15" s="38" t="n">
-        <v>557.7922360437625</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J15" s="38" t="n">
-        <v>284.9320665759161</v>
+        <v>280.4306484980009</v>
       </c>
       <c r="K15" s="38" t="n">
-        <v>327.6368284806779</v>
+        <v>321.9545044445791</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
@@ -2732,16 +2732,16 @@
         <v>1.645</v>
       </c>
       <c r="H16" s="38" t="n">
-        <v>438.2915456617699</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I16" s="38" t="n">
-        <v>616.1248789951032</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J16" s="38" t="n">
-        <v>276.272199681273</v>
+        <v>270.8940465957654</v>
       </c>
       <c r="K16" s="38" t="n">
-        <v>347.4055330146063</v>
+        <v>340.0603445585201</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
@@ -2786,16 +2786,16 @@
         <v>1.645</v>
       </c>
       <c r="H17" s="38" t="n">
-        <v>421.5024714616814</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I17" s="38" t="n">
-        <v>485.5262809854909</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J17" s="38" t="n">
-        <v>266.4567143423451</v>
+        <v>262.5414271293393</v>
       </c>
       <c r="K17" s="38" t="n">
-        <v>292.0662381518689</v>
+        <v>287.4427760678648</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
@@ -2840,16 +2840,16 @@
         <v>1.645</v>
       </c>
       <c r="H18" s="38" t="n">
-        <v>416.2999334681134</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I18" s="38" t="n">
-        <v>543.4427906109705</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J18" s="38" t="n">
-        <v>262.7922972752859</v>
+        <v>258.3113518538776</v>
       </c>
       <c r="K18" s="38" t="n">
-        <v>313.6494401324287</v>
+        <v>307.7621526466356</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
@@ -2894,16 +2894,16 @@
         <v>1.645</v>
       </c>
       <c r="H19" s="38" t="n">
-        <v>354.0146319193992</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I19" s="38" t="n">
-        <v>465.4193938241611</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J19" s="38" t="n">
-        <v>223.4480625268586</v>
+        <v>219.5946289031207</v>
       </c>
       <c r="K19" s="38" t="n">
-        <v>268.0099672887634</v>
+        <v>262.9242725190973</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
@@ -2948,16 +2948,16 @@
         <v>1.645</v>
       </c>
       <c r="H20" s="38" t="n">
-        <v>315.150722741428</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I20" s="38" t="n">
-        <v>389.4364370271423</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J20" s="38" t="n">
-        <v>199.093933051155</v>
+        <v>195.9517358949221</v>
       </c>
       <c r="K20" s="38" t="n">
-        <v>228.8082187654407</v>
+        <v>224.8443386052976</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
@@ -3002,16 +3002,16 @@
         <v>1.645</v>
       </c>
       <c r="H21" s="38" t="n">
-        <v>286.7725717849715</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I21" s="38" t="n">
-        <v>380.4868574992573</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J21" s="38" t="n">
-        <v>180.9773779721285</v>
+        <v>177.8089517637079</v>
       </c>
       <c r="K21" s="38" t="n">
-        <v>218.4630922578428</v>
+        <v>214.258081336797</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
@@ -3056,16 +3056,16 @@
         <v>1.645</v>
       </c>
       <c r="H22" s="38" t="n">
-        <v>283.0581654044113</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I22" s="38" t="n">
-        <v>343.5819749282209</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J22" s="38" t="n">
-        <v>178.8555138876847</v>
+        <v>176.0917866399555</v>
       </c>
       <c r="K22" s="38" t="n">
-        <v>203.0650376972085</v>
+        <v>199.6318494892422</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
@@ -3110,16 +3110,16 @@
         <v>1.645</v>
       </c>
       <c r="H23" s="38" t="n">
-        <v>274.3012574093693</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I23" s="38" t="n">
-        <v>344.2774478855598</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J23" s="38" t="n">
-        <v>173.2540588351115</v>
+        <v>170.464292326065</v>
       </c>
       <c r="K23" s="38" t="n">
-        <v>201.2445350255877</v>
+        <v>197.6807536612553</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
@@ -3145,39 +3145,39 @@
     <row r="24">
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>4200008229</t>
+          <t>4200009002</t>
         </is>
       </c>
       <c r="C24" s="38" t="n">
-        <v>801.1428571428571</v>
+        <v>427.7142857142857</v>
       </c>
       <c r="D24" s="38" t="n">
-        <v>387.7049688321558</v>
+        <v>389.2581466866233</v>
       </c>
       <c r="E24" s="38" t="n">
-        <v>26.7047619047619</v>
+        <v>14.25714285714286</v>
       </c>
       <c r="F24" s="38" t="n">
-        <v>70.78491902873635</v>
+        <v>71.06848921097281</v>
       </c>
       <c r="G24" s="38" t="n">
         <v>1.645</v>
       </c>
       <c r="H24" s="38" t="n">
-        <v>264.0502642846202</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I24" s="38" t="n">
-        <v>397.5740738084297</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J24" s="38" t="n">
-        <v>166.1311195364807</v>
+        <v>163.0304280298312</v>
       </c>
       <c r="K24" s="38" t="n">
-        <v>219.5406433460045</v>
+        <v>190.7562140922877</v>
       </c>
       <c r="L24" s="12" t="inlineStr">
         <is>
-          <t>Quạt treo ASIAvina - VY377990 - Xám</t>
+          <t>QUẠT treo ASIAVINA TURBO VY627890</t>
         </is>
       </c>
       <c r="M24" s="12" t="inlineStr">
@@ -3199,39 +3199,39 @@
     <row r="25">
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>4200009002</t>
+          <t>4200008229</t>
         </is>
       </c>
       <c r="C25" s="38" t="n">
-        <v>427.7142857142857</v>
+        <v>801.1428571428571</v>
       </c>
       <c r="D25" s="38" t="n">
-        <v>389.2581466866233</v>
+        <v>387.7049688321558</v>
       </c>
       <c r="E25" s="38" t="n">
-        <v>14.25714285714286</v>
+        <v>26.7047619047619</v>
       </c>
       <c r="F25" s="38" t="n">
-        <v>71.06848921097281</v>
+        <v>70.78491902873635</v>
       </c>
       <c r="G25" s="38" t="n">
         <v>1.645</v>
       </c>
       <c r="H25" s="38" t="n">
-        <v>262.4634328775895</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I25" s="38" t="n">
-        <v>333.7491471633037</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J25" s="38" t="n">
-        <v>165.7477449554158</v>
+        <v>162.3799207698659</v>
       </c>
       <c r="K25" s="38" t="n">
-        <v>194.2620306697015</v>
+        <v>214.3125220518485</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>QUẠT treo ASIAVINA TURBO VY627890</t>
+          <t>Quạt treo ASIAvina - VY377990 - Xám</t>
         </is>
       </c>
       <c r="M25" s="12" t="inlineStr">
@@ -3272,16 +3272,16 @@
         <v>1.645</v>
       </c>
       <c r="H26" s="38" t="n">
-        <v>258.0106686115152</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I26" s="38" t="n">
-        <v>346.2249543258009</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J26" s="38" t="n">
-        <v>162.7926786468204</v>
+        <v>159.887033795052</v>
       </c>
       <c r="K26" s="38" t="n">
-        <v>198.0783929325347</v>
+        <v>194.1969995136229</v>
       </c>
       <c r="L26" s="12" t="inlineStr">
         <is>
@@ -3326,16 +3326,16 @@
         <v>1.645</v>
       </c>
       <c r="H27" s="38" t="n">
-        <v>235.9010373926839</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I27" s="38" t="n">
-        <v>303.4724659641125</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J27" s="38" t="n">
-        <v>148.9482701243213</v>
+        <v>146.4648626696887</v>
       </c>
       <c r="K27" s="38" t="n">
-        <v>175.9768415528927</v>
+        <v>172.7460185966264</v>
       </c>
       <c r="L27" s="12" t="inlineStr">
         <is>
@@ -3380,16 +3380,16 @@
         <v>1.645</v>
       </c>
       <c r="H28" s="38" t="n">
-        <v>230.3812598278365</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I28" s="38" t="n">
-        <v>310.2622122087889</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J28" s="38" t="n">
-        <v>145.349948819531</v>
+        <v>142.7392804342588</v>
       </c>
       <c r="K28" s="38" t="n">
-        <v>177.302329771912</v>
+        <v>173.8080887974991</v>
       </c>
       <c r="L28" s="12" t="inlineStr">
         <is>
@@ -3434,16 +3434,16 @@
         <v>1.645</v>
       </c>
       <c r="H29" s="38" t="n">
-        <v>216.4386485788499</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I29" s="38" t="n">
-        <v>312.4624581026595</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J29" s="38" t="n">
-        <v>136.3399018976154</v>
+        <v>133.5362560796646</v>
       </c>
       <c r="K29" s="38" t="n">
-        <v>174.7494257071392</v>
+        <v>170.8836492626596</v>
       </c>
       <c r="L29" s="12" t="inlineStr">
         <is>
@@ -3488,16 +3488,16 @@
         <v>1.645</v>
       </c>
       <c r="H30" s="38" t="n">
-        <v>206.9246127460702</v>
+        <v>1.94469441319835</v>
       </c>
       <c r="I30" s="38" t="n">
-        <v>268.4960413174987</v>
+        <v>1.394523005618176</v>
       </c>
       <c r="J30" s="38" t="n">
-        <v>130.635241174403</v>
+        <v>128.4286025411084</v>
       </c>
       <c r="K30" s="38" t="n">
-        <v>155.2638126029744</v>
+        <v>152.3761251722081</v>
       </c>
       <c r="L30" s="12" t="inlineStr">
         <is>
@@ -3535,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D8"/>
+  <dimension ref="B1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3564,78 +3564,89 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>delta_from_lt2</t>
+          <t>delta_from_actual</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="38" t="n">
-        <v>12340.20950413805</v>
+        <v>8725.845821638699</v>
       </c>
       <c r="D3" s="38" t="n">
-        <v>0</v>
+        <v>-3442.546920113698</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="38" t="n">
-        <v>15113.60830209082</v>
+        <v>12340.20950413805</v>
       </c>
       <c r="D4" s="38" t="n">
-        <v>2773.398797952768</v>
+        <v>171.8167623856552</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="38" t="n">
-        <v>17451.6916432774</v>
+        <v>15113.60830209082</v>
       </c>
       <c r="D5" s="38" t="n">
-        <v>5111.482139139345</v>
+        <v>2945.215560338424</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" s="38" t="n">
-        <v>19511.58441836664</v>
+        <v>17451.6916432774</v>
       </c>
       <c r="D6" s="38" t="n">
-        <v>7171.374914228585</v>
+        <v>5283.298901525</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" s="38" t="n">
-        <v>21373.86983721144</v>
+        <v>19511.58441836664</v>
       </c>
       <c r="D7" s="38" t="n">
-        <v>9033.660333073392</v>
+        <v>7343.19167661424</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>21373.86983721144</v>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>9205.477095459048</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="37" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C9" s="38" t="n">
         <v>23086.41802274807</v>
       </c>
-      <c r="D8" s="38" t="n">
-        <v>10746.20851861002</v>
+      <c r="D9" s="38" t="n">
+        <v>10918.02528099567</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:D8"/>
+  <autoFilter ref="B2:D9"/>
   <mergeCells count="1">
     <mergeCell ref="B1:D1"/>
   </mergeCells>
@@ -3649,7 +3660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E4"/>
+  <dimension ref="B1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3724,8 +3735,26 @@
         <v>0.4874837261314043</v>
       </c>
     </row>
+    <row r="5">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Pooled (Mile-Weighted)</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Z * sigma * sqrt(1.9447)</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="n">
+        <v>12168.3927417524</v>
+      </c>
+      <c r="E5" s="38" t="n">
+        <v>0.6179683702789847</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B2:E4"/>
+  <autoFilter ref="B2:E5"/>
   <mergeCells count="1">
     <mergeCell ref="B1:E1"/>
   </mergeCells>

</xml_diff>